<commit_message>
fix: populate shared survey and BHA context in hydraulics workbook
</commit_message>
<xml_diff>
--- a/workbooks/source/Steady_State_Hydraulics_and_Nozzle_Optimization_SI.xlsx
+++ b/workbooks/source/Steady_State_Hydraulics_and_Nozzle_Optimization_SI.xlsx
@@ -4,23 +4,24 @@
   <x:sheets>
     <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="rId5"/>
     <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Inputs" sheetId="2" r:id="rId16"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Survey" sheetId="3" r:id="rId17"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Results" sheetId="4" r:id="rId18"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Graphs" sheetId="5" r:id="rId19"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fluid Model" sheetId="6" r:id="rId20"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Flow Path" sheetId="7" r:id="rId21"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Nozzle Cases" sheetId="8" r:id="rId22"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pressure Profile" sheetId="9" r:id="rId23"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Survey" sheetId="3" r:id="rId18"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Results" sheetId="4" r:id="rId19"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Graphs" sheetId="5" r:id="rId20"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fluid Model" sheetId="6" r:id="rId21"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Flow Path" sheetId="7" r:id="rId22"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Nozzle Cases" sheetId="8" r:id="rId23"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pressure Profile" sheetId="9" r:id="rId24"/>
     <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hydraulics Charts" sheetId="10" r:id="rId6"/>
     <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Flow Cases" sheetId="11" r:id="rId7"/>
     <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hydraulics Dashboard" sheetId="12" r:id="rId8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chart Settings" sheetId="13" r:id="rId9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Unit Map" sheetId="14" r:id="rId10"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checks" sheetId="15" r:id="rId11"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Calc" sheetId="16" r:id="rId12" state="hidden"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Exchange Map" sheetId="17" r:id="rId13"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Exchange State" sheetId="18" r:id="rId14" state="hidden"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Exchange Buffer" sheetId="19" r:id="rId15"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BHA Assembly" sheetId="13" r:id="rId9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chart Settings" sheetId="14" r:id="rId10"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Unit Map" sheetId="15" r:id="rId11"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checks" sheetId="16" r:id="rId12"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Calc" sheetId="17" r:id="rId13" state="hidden"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Exchange Map" sheetId="18" r:id="rId14"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Exchange State" sheetId="19" r:id="rId15" state="hidden"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Exchange Buffer" sheetId="20" r:id="rId17"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -3734,15 +3735,15 @@
       </x:c>
       <x:c r="B25" s="35" t="str">
         <x:f>"Static mud density "&amp;'Unit Map'!$H$13</x:f>
-        <x:v>Static mud density kg/m3</x:v>
+        <x:v>Static mud density g/cm3</x:v>
       </x:c>
       <x:c r="C25" s="35" t="str">
         <x:f>"ECD "&amp;'Unit Map'!$H$13</x:f>
-        <x:v>ECD kg/m3</x:v>
+        <x:v>ECD g/cm3</x:v>
       </x:c>
       <x:c r="D25" s="35" t="str">
         <x:f>"ECD screen "&amp;'Unit Map'!$H$13</x:f>
-        <x:v>ECD screen kg/m3</x:v>
+        <x:v>ECD screen g/cm3</x:v>
       </x:c>
       <x:c r="E25" s="35"/>
       <x:c r="F25" s="35"/>
@@ -3762,15 +3763,15 @@
       </x:c>
       <x:c r="B26" s="35" t="n">
         <x:f>'Inputs'!$B$9*'Unit Map'!$I$13</x:f>
-        <x:v>1200</x:v>
+        <x:v>1.2</x:v>
       </x:c>
       <x:c r="C26" s="35" t="n">
         <x:f>'Pressure Profile'!H6</x:f>
-        <x:v>1200</x:v>
+        <x:v>1.2</x:v>
       </x:c>
       <x:c r="D26" s="35" t="n">
         <x:f>'Inputs'!$B$14*'Unit Map'!$I$13</x:f>
-        <x:v>1400</x:v>
+        <x:v>1.4000000000000001</x:v>
       </x:c>
       <x:c r="E26" s="35"/>
       <x:c r="F26" s="35"/>
@@ -3790,15 +3791,15 @@
       </x:c>
       <x:c r="B27" s="35" t="n">
         <x:f>'Inputs'!$B$9*'Unit Map'!$I$13</x:f>
-        <x:v>1200</x:v>
+        <x:v>1.2</x:v>
       </x:c>
       <x:c r="C27" s="35" t="n">
         <x:f>'Pressure Profile'!H7</x:f>
-        <x:v>1200</x:v>
+        <x:v>1.2</x:v>
       </x:c>
       <x:c r="D27" s="35" t="n">
         <x:f>'Inputs'!$B$14*'Unit Map'!$I$13</x:f>
-        <x:v>1400</x:v>
+        <x:v>1.4000000000000001</x:v>
       </x:c>
       <x:c r="E27" s="35"/>
       <x:c r="F27" s="35"/>
@@ -3818,15 +3819,15 @@
       </x:c>
       <x:c r="B28" s="35" t="n">
         <x:f>'Inputs'!$B$9*'Unit Map'!$I$13</x:f>
-        <x:v>1200</x:v>
+        <x:v>1.2</x:v>
       </x:c>
       <x:c r="C28" s="35" t="n">
         <x:f>'Pressure Profile'!H8</x:f>
-        <x:v>1200</x:v>
+        <x:v>1.2</x:v>
       </x:c>
       <x:c r="D28" s="35" t="n">
         <x:f>'Inputs'!$B$14*'Unit Map'!$I$13</x:f>
-        <x:v>1400</x:v>
+        <x:v>1.4000000000000001</x:v>
       </x:c>
       <x:c r="E28" s="35"/>
       <x:c r="F28" s="35"/>
@@ -3846,15 +3847,15 @@
       </x:c>
       <x:c r="B29" s="35" t="n">
         <x:f>'Inputs'!$B$9*'Unit Map'!$I$13</x:f>
-        <x:v>1200</x:v>
+        <x:v>1.2</x:v>
       </x:c>
       <x:c r="C29" s="35" t="n">
         <x:f>'Pressure Profile'!H9</x:f>
-        <x:v>1200</x:v>
+        <x:v>1.2</x:v>
       </x:c>
       <x:c r="D29" s="35" t="n">
         <x:f>'Inputs'!$B$14*'Unit Map'!$I$13</x:f>
-        <x:v>1400</x:v>
+        <x:v>1.4000000000000001</x:v>
       </x:c>
       <x:c r="E29" s="35"/>
       <x:c r="F29" s="35"/>
@@ -3874,15 +3875,15 @@
       </x:c>
       <x:c r="B30" s="35" t="n">
         <x:f>'Inputs'!$B$9*'Unit Map'!$I$13</x:f>
-        <x:v>1200</x:v>
+        <x:v>1.2</x:v>
       </x:c>
       <x:c r="C30" s="35" t="n">
         <x:f>'Pressure Profile'!H10</x:f>
-        <x:v>1200</x:v>
+        <x:v>1.2</x:v>
       </x:c>
       <x:c r="D30" s="35" t="n">
         <x:f>'Inputs'!$B$14*'Unit Map'!$I$13</x:f>
-        <x:v>1400</x:v>
+        <x:v>1.4000000000000001</x:v>
       </x:c>
       <x:c r="E30" s="35"/>
       <x:c r="F30" s="35"/>
@@ -3902,15 +3903,15 @@
       </x:c>
       <x:c r="B31" s="35" t="n">
         <x:f>'Inputs'!$B$9*'Unit Map'!$I$13</x:f>
-        <x:v>1200</x:v>
+        <x:v>1.2</x:v>
       </x:c>
       <x:c r="C31" s="35" t="n">
         <x:f>'Pressure Profile'!H11</x:f>
-        <x:v>1200</x:v>
+        <x:v>1.2</x:v>
       </x:c>
       <x:c r="D31" s="35" t="n">
         <x:f>'Inputs'!$B$14*'Unit Map'!$I$13</x:f>
-        <x:v>1400</x:v>
+        <x:v>1.4000000000000001</x:v>
       </x:c>
       <x:c r="E31" s="35"/>
       <x:c r="F31" s="35"/>
@@ -3930,15 +3931,15 @@
       </x:c>
       <x:c r="B32" s="35" t="n">
         <x:f>'Inputs'!$B$9*'Unit Map'!$I$13</x:f>
-        <x:v>1200</x:v>
+        <x:v>1.2</x:v>
       </x:c>
       <x:c r="C32" s="35" t="n">
         <x:f>'Pressure Profile'!H12</x:f>
-        <x:v>1200</x:v>
+        <x:v>1.2</x:v>
       </x:c>
       <x:c r="D32" s="35" t="n">
         <x:f>'Inputs'!$B$14*'Unit Map'!$I$13</x:f>
-        <x:v>1400</x:v>
+        <x:v>1.4000000000000001</x:v>
       </x:c>
       <x:c r="E32" s="35"/>
       <x:c r="F32" s="35"/>
@@ -3958,15 +3959,15 @@
       </x:c>
       <x:c r="B33" s="35" t="n">
         <x:f>'Inputs'!$B$9*'Unit Map'!$I$13</x:f>
-        <x:v>1200</x:v>
+        <x:v>1.2</x:v>
       </x:c>
       <x:c r="C33" s="35" t="n">
         <x:f>'Pressure Profile'!H13</x:f>
-        <x:v>1769.9514042766855</x:v>
+        <x:v>1.7699514042766855</x:v>
       </x:c>
       <x:c r="D33" s="35" t="n">
         <x:f>'Inputs'!$B$14*'Unit Map'!$I$13</x:f>
-        <x:v>1400</x:v>
+        <x:v>1.4000000000000001</x:v>
       </x:c>
       <x:c r="E33" s="35"/>
       <x:c r="F33" s="35"/>
@@ -5324,7 +5325,7 @@
       </x:c>
       <x:c r="B12" s="37" t="n">
         <x:f>INDEX($J$46:$J$53,MATCH($B$5,$H$46:$H$53,1))</x:f>
-        <x:v>1200</x:v>
+        <x:v>1.2</x:v>
       </x:c>
       <x:c r="C12" s="35"/>
       <x:c r="D12" s="35"/>
@@ -5356,7 +5357,7 @@
       </x:c>
       <x:c r="B13" s="37" t="n">
         <x:f>INDEX($M$46:$M$53,MATCH($B$5,$H$46:$H$53,1))-INDEX($J$46:$J$53,MATCH($B$5,$H$46:$H$53,1))</x:f>
-        <x:v>200</x:v>
+        <x:v>0.20000000000000018</x:v>
       </x:c>
       <x:c r="C13" s="35"/>
       <x:c r="D13" s="35"/>
@@ -6296,23 +6297,23 @@
       </x:c>
       <x:c r="I45" s="35" t="str">
         <x:f>"Low flow ECD "&amp;'Unit Map'!$H$13</x:f>
-        <x:v>Low flow ECD kg/m3</x:v>
+        <x:v>Low flow ECD g/cm3</x:v>
       </x:c>
       <x:c r="J45" s="35" t="str">
         <x:f>"Base flow ECD "&amp;'Unit Map'!$H$13</x:f>
-        <x:v>Base flow ECD kg/m3</x:v>
+        <x:v>Base flow ECD g/cm3</x:v>
       </x:c>
       <x:c r="K45" s="35" t="str">
         <x:f>"High flow ECD "&amp;'Unit Map'!$H$13</x:f>
-        <x:v>High flow ECD kg/m3</x:v>
+        <x:v>High flow ECD g/cm3</x:v>
       </x:c>
       <x:c r="L45" s="35" t="str">
         <x:f>"Static density "&amp;'Unit Map'!$H$13</x:f>
-        <x:v>Static density kg/m3</x:v>
+        <x:v>Static density g/cm3</x:v>
       </x:c>
       <x:c r="M45" s="35" t="str">
         <x:f>"ECD limit "&amp;'Unit Map'!$H$13</x:f>
-        <x:v>ECD limit kg/m3</x:v>
+        <x:v>ECD limit g/cm3</x:v>
       </x:c>
       <x:c r="N45" s="35"/>
       <x:c r="O45" s="35" t="str">
@@ -6386,23 +6387,23 @@
       </x:c>
       <x:c r="I46" s="35" t="n">
         <x:f>('Inputs'!$B$9+('Pressure Profile'!H6/'Unit Map'!$I$13-'Inputs'!$B$9)*'Flow Cases'!B6^1.75)*'Unit Map'!$I$13</x:f>
-        <x:v>1200</x:v>
+        <x:v>1.2</x:v>
       </x:c>
       <x:c r="J46" s="35" t="n">
         <x:f>'Pressure Profile'!H6</x:f>
-        <x:v>1200</x:v>
+        <x:v>1.2</x:v>
       </x:c>
       <x:c r="K46" s="35" t="n">
         <x:f>('Inputs'!$B$9+('Pressure Profile'!H6/'Unit Map'!$I$13-'Inputs'!$B$9)*'Flow Cases'!B8^1.75)*'Unit Map'!$I$13</x:f>
-        <x:v>1200</x:v>
+        <x:v>1.2</x:v>
       </x:c>
       <x:c r="L46" s="35" t="n">
         <x:f>'Inputs'!$B$9*'Unit Map'!$I$13</x:f>
-        <x:v>1200</x:v>
+        <x:v>1.2</x:v>
       </x:c>
       <x:c r="M46" s="35" t="n">
         <x:f>'Inputs'!$B$14*'Unit Map'!$I$13</x:f>
-        <x:v>1400</x:v>
+        <x:v>1.4000000000000001</x:v>
       </x:c>
       <x:c r="N46" s="35"/>
       <x:c r="O46" s="35" t="n">
@@ -6476,23 +6477,23 @@
       </x:c>
       <x:c r="I47" s="35" t="n">
         <x:f>('Inputs'!$B$9+('Pressure Profile'!H7/'Unit Map'!$I$13-'Inputs'!$B$9)*'Flow Cases'!B6^1.75)*'Unit Map'!$I$13</x:f>
-        <x:v>1200</x:v>
+        <x:v>1.2</x:v>
       </x:c>
       <x:c r="J47" s="35" t="n">
         <x:f>'Pressure Profile'!H7</x:f>
-        <x:v>1200</x:v>
+        <x:v>1.2</x:v>
       </x:c>
       <x:c r="K47" s="35" t="n">
         <x:f>('Inputs'!$B$9+('Pressure Profile'!H7/'Unit Map'!$I$13-'Inputs'!$B$9)*'Flow Cases'!B8^1.75)*'Unit Map'!$I$13</x:f>
-        <x:v>1200</x:v>
+        <x:v>1.2</x:v>
       </x:c>
       <x:c r="L47" s="35" t="n">
         <x:f>'Inputs'!$B$9*'Unit Map'!$I$13</x:f>
-        <x:v>1200</x:v>
+        <x:v>1.2</x:v>
       </x:c>
       <x:c r="M47" s="35" t="n">
         <x:f>'Inputs'!$B$14*'Unit Map'!$I$13</x:f>
-        <x:v>1400</x:v>
+        <x:v>1.4000000000000001</x:v>
       </x:c>
       <x:c r="N47" s="35"/>
       <x:c r="O47" s="35" t="n">
@@ -6566,23 +6567,23 @@
       </x:c>
       <x:c r="I48" s="35" t="n">
         <x:f>('Inputs'!$B$9+('Pressure Profile'!H8/'Unit Map'!$I$13-'Inputs'!$B$9)*'Flow Cases'!B6^1.75)*'Unit Map'!$I$13</x:f>
-        <x:v>1200</x:v>
+        <x:v>1.2</x:v>
       </x:c>
       <x:c r="J48" s="35" t="n">
         <x:f>'Pressure Profile'!H8</x:f>
-        <x:v>1200</x:v>
+        <x:v>1.2</x:v>
       </x:c>
       <x:c r="K48" s="35" t="n">
         <x:f>('Inputs'!$B$9+('Pressure Profile'!H8/'Unit Map'!$I$13-'Inputs'!$B$9)*'Flow Cases'!B8^1.75)*'Unit Map'!$I$13</x:f>
-        <x:v>1200</x:v>
+        <x:v>1.2</x:v>
       </x:c>
       <x:c r="L48" s="35" t="n">
         <x:f>'Inputs'!$B$9*'Unit Map'!$I$13</x:f>
-        <x:v>1200</x:v>
+        <x:v>1.2</x:v>
       </x:c>
       <x:c r="M48" s="35" t="n">
         <x:f>'Inputs'!$B$14*'Unit Map'!$I$13</x:f>
-        <x:v>1400</x:v>
+        <x:v>1.4000000000000001</x:v>
       </x:c>
       <x:c r="N48" s="35"/>
       <x:c r="O48" s="35" t="n">
@@ -6656,23 +6657,23 @@
       </x:c>
       <x:c r="I49" s="35" t="n">
         <x:f>('Inputs'!$B$9+('Pressure Profile'!H9/'Unit Map'!$I$13-'Inputs'!$B$9)*'Flow Cases'!B6^1.75)*'Unit Map'!$I$13</x:f>
-        <x:v>1200</x:v>
+        <x:v>1.2</x:v>
       </x:c>
       <x:c r="J49" s="35" t="n">
         <x:f>'Pressure Profile'!H9</x:f>
-        <x:v>1200</x:v>
+        <x:v>1.2</x:v>
       </x:c>
       <x:c r="K49" s="35" t="n">
         <x:f>('Inputs'!$B$9+('Pressure Profile'!H9/'Unit Map'!$I$13-'Inputs'!$B$9)*'Flow Cases'!B8^1.75)*'Unit Map'!$I$13</x:f>
-        <x:v>1200</x:v>
+        <x:v>1.2</x:v>
       </x:c>
       <x:c r="L49" s="35" t="n">
         <x:f>'Inputs'!$B$9*'Unit Map'!$I$13</x:f>
-        <x:v>1200</x:v>
+        <x:v>1.2</x:v>
       </x:c>
       <x:c r="M49" s="35" t="n">
         <x:f>'Inputs'!$B$14*'Unit Map'!$I$13</x:f>
-        <x:v>1400</x:v>
+        <x:v>1.4000000000000001</x:v>
       </x:c>
       <x:c r="N49" s="35"/>
       <x:c r="O49" s="35" t="n">
@@ -6746,23 +6747,23 @@
       </x:c>
       <x:c r="I50" s="35" t="n">
         <x:f>('Inputs'!$B$9+('Pressure Profile'!H10/'Unit Map'!$I$13-'Inputs'!$B$9)*'Flow Cases'!B6^1.75)*'Unit Map'!$I$13</x:f>
-        <x:v>1200</x:v>
+        <x:v>1.2</x:v>
       </x:c>
       <x:c r="J50" s="35" t="n">
         <x:f>'Pressure Profile'!H10</x:f>
-        <x:v>1200</x:v>
+        <x:v>1.2</x:v>
       </x:c>
       <x:c r="K50" s="35" t="n">
         <x:f>('Inputs'!$B$9+('Pressure Profile'!H10/'Unit Map'!$I$13-'Inputs'!$B$9)*'Flow Cases'!B8^1.75)*'Unit Map'!$I$13</x:f>
-        <x:v>1200</x:v>
+        <x:v>1.2</x:v>
       </x:c>
       <x:c r="L50" s="35" t="n">
         <x:f>'Inputs'!$B$9*'Unit Map'!$I$13</x:f>
-        <x:v>1200</x:v>
+        <x:v>1.2</x:v>
       </x:c>
       <x:c r="M50" s="35" t="n">
         <x:f>'Inputs'!$B$14*'Unit Map'!$I$13</x:f>
-        <x:v>1400</x:v>
+        <x:v>1.4000000000000001</x:v>
       </x:c>
       <x:c r="N50" s="35"/>
       <x:c r="O50" s="35" t="n">
@@ -6836,23 +6837,23 @@
       </x:c>
       <x:c r="I51" s="35" t="n">
         <x:f>('Inputs'!$B$9+('Pressure Profile'!H11/'Unit Map'!$I$13-'Inputs'!$B$9)*'Flow Cases'!B6^1.75)*'Unit Map'!$I$13</x:f>
-        <x:v>1200</x:v>
+        <x:v>1.2</x:v>
       </x:c>
       <x:c r="J51" s="35" t="n">
         <x:f>'Pressure Profile'!H11</x:f>
-        <x:v>1200</x:v>
+        <x:v>1.2</x:v>
       </x:c>
       <x:c r="K51" s="35" t="n">
         <x:f>('Inputs'!$B$9+('Pressure Profile'!H11/'Unit Map'!$I$13-'Inputs'!$B$9)*'Flow Cases'!B8^1.75)*'Unit Map'!$I$13</x:f>
-        <x:v>1200</x:v>
+        <x:v>1.2</x:v>
       </x:c>
       <x:c r="L51" s="35" t="n">
         <x:f>'Inputs'!$B$9*'Unit Map'!$I$13</x:f>
-        <x:v>1200</x:v>
+        <x:v>1.2</x:v>
       </x:c>
       <x:c r="M51" s="35" t="n">
         <x:f>'Inputs'!$B$14*'Unit Map'!$I$13</x:f>
-        <x:v>1400</x:v>
+        <x:v>1.4000000000000001</x:v>
       </x:c>
       <x:c r="N51" s="35"/>
       <x:c r="O51" s="35" t="n">
@@ -6914,23 +6915,23 @@
       </x:c>
       <x:c r="I52" s="35" t="n">
         <x:f>('Inputs'!$B$9+('Pressure Profile'!H12/'Unit Map'!$I$13-'Inputs'!$B$9)*'Flow Cases'!B6^1.75)*'Unit Map'!$I$13</x:f>
-        <x:v>1200</x:v>
+        <x:v>1.2</x:v>
       </x:c>
       <x:c r="J52" s="35" t="n">
         <x:f>'Pressure Profile'!H12</x:f>
-        <x:v>1200</x:v>
+        <x:v>1.2</x:v>
       </x:c>
       <x:c r="K52" s="35" t="n">
         <x:f>('Inputs'!$B$9+('Pressure Profile'!H12/'Unit Map'!$I$13-'Inputs'!$B$9)*'Flow Cases'!B8^1.75)*'Unit Map'!$I$13</x:f>
-        <x:v>1200</x:v>
+        <x:v>1.2</x:v>
       </x:c>
       <x:c r="L52" s="35" t="n">
         <x:f>'Inputs'!$B$9*'Unit Map'!$I$13</x:f>
-        <x:v>1200</x:v>
+        <x:v>1.2</x:v>
       </x:c>
       <x:c r="M52" s="35" t="n">
         <x:f>'Inputs'!$B$14*'Unit Map'!$I$13</x:f>
-        <x:v>1400</x:v>
+        <x:v>1.4000000000000001</x:v>
       </x:c>
       <x:c r="N52" s="35"/>
       <x:c r="O52" s="35" t="n">
@@ -6992,23 +6993,23 @@
       </x:c>
       <x:c r="I53" s="35" t="n">
         <x:f>('Inputs'!$B$9+('Pressure Profile'!H13/'Unit Map'!$I$13-'Inputs'!$B$9)*'Flow Cases'!B6^1.75)*'Unit Map'!$I$13</x:f>
-        <x:v>1628.8653391588261</x:v>
+        <x:v>1.6288653391588261</x:v>
       </x:c>
       <x:c r="J53" s="35" t="n">
         <x:f>'Pressure Profile'!H13</x:f>
-        <x:v>1769.9514042766855</x:v>
+        <x:v>1.7699514042766855</x:v>
       </x:c>
       <x:c r="K53" s="35" t="n">
         <x:f>('Inputs'!$B$9+('Pressure Profile'!H13/'Unit Map'!$I$13-'Inputs'!$B$9)*'Flow Cases'!B8^1.75)*'Unit Map'!$I$13</x:f>
-        <x:v>1927.8787635153908</x:v>
+        <x:v>1.927878763515391</x:v>
       </x:c>
       <x:c r="L53" s="35" t="n">
         <x:f>'Inputs'!$B$9*'Unit Map'!$I$13</x:f>
-        <x:v>1200</x:v>
+        <x:v>1.2</x:v>
       </x:c>
       <x:c r="M53" s="35" t="n">
         <x:f>'Inputs'!$B$14*'Unit Map'!$I$13</x:f>
-        <x:v>1400</x:v>
+        <x:v>1.4000000000000001</x:v>
       </x:c>
       <x:c r="N53" s="35"/>
       <x:c r="O53" s="35" t="n">
@@ -7049,6 +7050,487 @@
 </file>
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="22" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="12" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="12" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="12" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="12" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="12" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="12" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="12" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="12" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="12" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="12" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="12" hidden="0" customWidth="1"/>
+    <x:col min="13" max="13" width="12" hidden="0" customWidth="1"/>
+    <x:col min="14" max="14" width="12" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="26" customHeight="1">
+      <x:c r="A1" s="34" t="str">
+        <x:v>WellForge | BHA Assembly | Formula-driven planning and review workbook</x:v>
+      </x:c>
+      <x:c r="B1" s="34"/>
+      <x:c r="C1" s="34"/>
+      <x:c r="D1" s="34"/>
+      <x:c r="E1" s="34"/>
+      <x:c r="F1" s="34"/>
+      <x:c r="G1" s="34"/>
+      <x:c r="H1" s="34"/>
+      <x:c r="I1" s="34"/>
+      <x:c r="J1" s="34"/>
+      <x:c r="K1" s="34"/>
+      <x:c r="L1" s="34"/>
+      <x:c r="M1" s="34"/>
+      <x:c r="N1" s="34"/>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" s="35"/>
+      <x:c r="B2" s="35"/>
+      <x:c r="C2" s="35"/>
+      <x:c r="D2" s="35"/>
+      <x:c r="E2" s="35"/>
+      <x:c r="F2" s="35"/>
+      <x:c r="G2" s="35"/>
+      <x:c r="H2" s="35"/>
+      <x:c r="I2" s="35"/>
+      <x:c r="J2" s="35"/>
+      <x:c r="K2" s="35"/>
+      <x:c r="L2" s="35"/>
+      <x:c r="M2" s="35"/>
+      <x:c r="N2" s="35"/>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" s="38" t="str">
+        <x:v>Shared SI BHA assembly — reused by hydraulics, torque/drag and BHA models</x:v>
+      </x:c>
+      <x:c r="B3" s="38" t="str">
+        <x:v>Shared SI BHA assembly — reused by hydraulics, torque/drag and BHA models</x:v>
+      </x:c>
+      <x:c r="C3" s="38" t="str">
+        <x:v>Shared SI BHA assembly — reused by hydraulics, torque/drag and BHA models</x:v>
+      </x:c>
+      <x:c r="D3" s="38" t="str">
+        <x:v>Shared SI BHA assembly — reused by hydraulics, torque/drag and BHA models</x:v>
+      </x:c>
+      <x:c r="E3" s="38" t="str">
+        <x:v>Shared SI BHA assembly — reused by hydraulics, torque/drag and BHA models</x:v>
+      </x:c>
+      <x:c r="F3" s="38" t="str">
+        <x:v>Shared SI BHA assembly — reused by hydraulics, torque/drag and BHA models</x:v>
+      </x:c>
+      <x:c r="G3" s="38" t="str">
+        <x:v>Shared SI BHA assembly — reused by hydraulics, torque/drag and BHA models</x:v>
+      </x:c>
+      <x:c r="H3" s="38" t="str">
+        <x:v>Shared SI BHA assembly — reused by hydraulics, torque/drag and BHA models</x:v>
+      </x:c>
+      <x:c r="I3" s="38" t="str">
+        <x:v>Shared SI BHA assembly — reused by hydraulics, torque/drag and BHA models</x:v>
+      </x:c>
+      <x:c r="J3" s="38" t="str">
+        <x:v>Shared SI BHA assembly — reused by hydraulics, torque/drag and BHA models</x:v>
+      </x:c>
+      <x:c r="K3" s="38" t="str">
+        <x:v>Shared SI BHA assembly — reused by hydraulics, torque/drag and BHA models</x:v>
+      </x:c>
+      <x:c r="L3" s="38" t="str">
+        <x:v>Shared SI BHA assembly — reused by hydraulics, torque/drag and BHA models</x:v>
+      </x:c>
+      <x:c r="M3" s="38" t="str">
+        <x:v>Shared SI BHA assembly — reused by hydraulics, torque/drag and BHA models</x:v>
+      </x:c>
+      <x:c r="N3" s="35"/>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" s="35"/>
+      <x:c r="B4" s="35"/>
+      <x:c r="C4" s="35"/>
+      <x:c r="D4" s="35"/>
+      <x:c r="E4" s="35"/>
+      <x:c r="F4" s="35"/>
+      <x:c r="G4" s="35"/>
+      <x:c r="H4" s="35"/>
+      <x:c r="I4" s="35"/>
+      <x:c r="J4" s="35"/>
+      <x:c r="K4" s="35"/>
+      <x:c r="L4" s="35"/>
+      <x:c r="M4" s="35"/>
+      <x:c r="N4" s="35"/>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" s="36" t="str">
+        <x:v>Record ID</x:v>
+      </x:c>
+      <x:c r="B5" s="36" t="str">
+        <x:v>Component</x:v>
+      </x:c>
+      <x:c r="C5" s="36" t="str">
+        <x:v>Top m</x:v>
+      </x:c>
+      <x:c r="D5" s="36" t="str">
+        <x:v>Bottom m</x:v>
+      </x:c>
+      <x:c r="E5" s="36" t="str">
+        <x:v>Length m</x:v>
+      </x:c>
+      <x:c r="F5" s="36" t="str">
+        <x:v>OD m</x:v>
+      </x:c>
+      <x:c r="G5" s="36" t="str">
+        <x:v>ID m</x:v>
+      </x:c>
+      <x:c r="H5" s="36" t="str">
+        <x:v>Area m2</x:v>
+      </x:c>
+      <x:c r="I5" s="36" t="str">
+        <x:v>I m4</x:v>
+      </x:c>
+      <x:c r="J5" s="36" t="str">
+        <x:v>Mass kg</x:v>
+      </x:c>
+      <x:c r="K5" s="36" t="str">
+        <x:v>Support factor</x:v>
+      </x:c>
+      <x:c r="L5" s="36" t="str">
+        <x:v>Connection / role</x:v>
+      </x:c>
+      <x:c r="M5" s="36" t="str">
+        <x:v>Status</x:v>
+      </x:c>
+      <x:c r="N5" s="35"/>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" s="37" t="str">
+        <x:v>bha-bit</x:v>
+      </x:c>
+      <x:c r="B6" s="37" t="str">
+        <x:v>Bit</x:v>
+      </x:c>
+      <x:c r="C6" s="37" t="n">
+        <x:f>0</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D6" s="37" t="n">
+        <x:f>C6+E6</x:f>
+        <x:v>0.3</x:v>
+      </x:c>
+      <x:c r="E6" s="37" t="n">
+        <x:f>0.3</x:f>
+        <x:v>0.3</x:v>
+      </x:c>
+      <x:c r="F6" s="37" t="n">
+        <x:f>0.216</x:f>
+        <x:v>0.216</x:v>
+      </x:c>
+      <x:c r="G6" s="37" t="n">
+        <x:f>0.05</x:f>
+        <x:v>0.05</x:v>
+      </x:c>
+      <x:c r="H6" s="37" t="n">
+        <x:f>PI()/4*(F6^2-G6^2)</x:f>
+        <x:v>0.03468004130297772</x:v>
+      </x:c>
+      <x:c r="I6" s="37" t="n">
+        <x:f>PI()/64*(F6^4-G6^4)</x:f>
+        <x:v>0.0001065457568930733</x:v>
+      </x:c>
+      <x:c r="J6" s="37" t="n">
+        <x:f>H6*E6*7850</x:f>
+        <x:v>81.67149726851254</x:v>
+      </x:c>
+      <x:c r="K6" s="37" t="n">
+        <x:f>1</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="L6" s="37" t="str">
+        <x:f>"Bit / formation interface"</x:f>
+        <x:v>Bit / formation interface</x:v>
+      </x:c>
+      <x:c r="M6" s="37" t="str">
+        <x:f>IF(AND(F6&gt;G6,E6&gt;0),"PASS","REVIEW")</x:f>
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="N6" s="35"/>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" s="37" t="str">
+        <x:v>bha-near-bit-stabilizer</x:v>
+      </x:c>
+      <x:c r="B7" s="37" t="str">
+        <x:v>Near-bit stabilizer</x:v>
+      </x:c>
+      <x:c r="C7" s="37" t="n">
+        <x:f>D6</x:f>
+        <x:v>0.3</x:v>
+      </x:c>
+      <x:c r="D7" s="37" t="n">
+        <x:f>C7+E7</x:f>
+        <x:v>1.8</x:v>
+      </x:c>
+      <x:c r="E7" s="37" t="n">
+        <x:f>1.5</x:f>
+        <x:v>1.5</x:v>
+      </x:c>
+      <x:c r="F7" s="37" t="n">
+        <x:f>0.203</x:f>
+        <x:v>0.203</x:v>
+      </x:c>
+      <x:c r="G7" s="37" t="n">
+        <x:f>0.07</x:f>
+        <x:v>0.07</x:v>
+      </x:c>
+      <x:c r="H7" s="37" t="n">
+        <x:f>PI()/4*(F7^2-G7^2)</x:f>
+        <x:v>0.02851702191479795</x:v>
+      </x:c>
+      <x:c r="I7" s="37" t="n">
+        <x:f>PI()/64*(F7^4-G7^4)</x:f>
+        <x:v>0.00008218071021683868</x:v>
+      </x:c>
+      <x:c r="J7" s="37" t="n">
+        <x:f>H7*E7*7850</x:f>
+        <x:v>335.7879330467459</x:v>
+      </x:c>
+      <x:c r="K7" s="37" t="n">
+        <x:f>0.85</x:f>
+        <x:v>0.85</x:v>
+      </x:c>
+      <x:c r="L7" s="37" t="str">
+        <x:f>"BHA component"</x:f>
+        <x:v>BHA component</x:v>
+      </x:c>
+      <x:c r="M7" s="37" t="str">
+        <x:f>IF(AND(F7&gt;G7,E7&gt;0),"PASS","REVIEW")</x:f>
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="N7" s="35"/>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" s="37" t="str">
+        <x:v>bha-motor-rss</x:v>
+      </x:c>
+      <x:c r="B8" s="37" t="str">
+        <x:v>Motor / RSS</x:v>
+      </x:c>
+      <x:c r="C8" s="37" t="n">
+        <x:f>D7</x:f>
+        <x:v>1.8</x:v>
+      </x:c>
+      <x:c r="D8" s="37" t="n">
+        <x:f>C8+E8</x:f>
+        <x:v>9.8</x:v>
+      </x:c>
+      <x:c r="E8" s="37" t="n">
+        <x:f>8</x:f>
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="F8" s="37" t="n">
+        <x:f>0.171</x:f>
+        <x:v>0.171</x:v>
+      </x:c>
+      <x:c r="G8" s="37" t="n">
+        <x:f>0.057</x:f>
+        <x:v>0.057</x:v>
+      </x:c>
+      <x:c r="H8" s="37" t="n">
+        <x:f>PI()/4*(F8^2-G8^2)</x:f>
+        <x:v>0.020414069063026476</x:v>
+      </x:c>
+      <x:c r="I8" s="37" t="n">
+        <x:f>PI()/64*(F8^4-G8^4)</x:f>
+        <x:v>0.00004145331899110815</x:v>
+      </x:c>
+      <x:c r="J8" s="37" t="n">
+        <x:f>H8*E8*7850</x:f>
+        <x:v>1282.0035371580627</x:v>
+      </x:c>
+      <x:c r="K8" s="37" t="n">
+        <x:f>0.7</x:f>
+        <x:v>0.7</x:v>
+      </x:c>
+      <x:c r="L8" s="37" t="str">
+        <x:f>"BHA component"</x:f>
+        <x:v>BHA component</x:v>
+      </x:c>
+      <x:c r="M8" s="37" t="str">
+        <x:f>IF(AND(F8&gt;G8,E8&gt;0),"PASS","REVIEW")</x:f>
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="N8" s="35"/>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" s="37" t="str">
+        <x:v>bha-mwd-lwd</x:v>
+      </x:c>
+      <x:c r="B9" s="37" t="str">
+        <x:v>MWD / LWD</x:v>
+      </x:c>
+      <x:c r="C9" s="37" t="n">
+        <x:f>D8</x:f>
+        <x:v>9.8</x:v>
+      </x:c>
+      <x:c r="D9" s="37" t="n">
+        <x:f>C9+E9</x:f>
+        <x:v>21.8</x:v>
+      </x:c>
+      <x:c r="E9" s="37" t="n">
+        <x:f>12</x:f>
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="F9" s="37" t="n">
+        <x:f>0.171</x:f>
+        <x:v>0.171</x:v>
+      </x:c>
+      <x:c r="G9" s="37" t="n">
+        <x:f>0.057</x:f>
+        <x:v>0.057</x:v>
+      </x:c>
+      <x:c r="H9" s="37" t="n">
+        <x:f>PI()/4*(F9^2-G9^2)</x:f>
+        <x:v>0.020414069063026476</x:v>
+      </x:c>
+      <x:c r="I9" s="37" t="n">
+        <x:f>PI()/64*(F9^4-G9^4)</x:f>
+        <x:v>0.00004145331899110815</x:v>
+      </x:c>
+      <x:c r="J9" s="37" t="n">
+        <x:f>H9*E9*7850</x:f>
+        <x:v>1923.005305737094</x:v>
+      </x:c>
+      <x:c r="K9" s="37" t="n">
+        <x:f>0.65</x:f>
+        <x:v>0.65</x:v>
+      </x:c>
+      <x:c r="L9" s="37" t="str">
+        <x:f>"BHA component"</x:f>
+        <x:v>BHA component</x:v>
+      </x:c>
+      <x:c r="M9" s="37" t="str">
+        <x:f>IF(AND(F9&gt;G9,E9&gt;0),"PASS","REVIEW")</x:f>
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="N9" s="35"/>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" s="37" t="str">
+        <x:v>bha-drill-collar</x:v>
+      </x:c>
+      <x:c r="B10" s="37" t="str">
+        <x:v>Drill collar</x:v>
+      </x:c>
+      <x:c r="C10" s="37" t="n">
+        <x:f>D9</x:f>
+        <x:v>21.8</x:v>
+      </x:c>
+      <x:c r="D10" s="37" t="n">
+        <x:f>C10+E10</x:f>
+        <x:v>111.8</x:v>
+      </x:c>
+      <x:c r="E10" s="37" t="n">
+        <x:f>90</x:f>
+        <x:v>90</x:v>
+      </x:c>
+      <x:c r="F10" s="37" t="n">
+        <x:f>0.171</x:f>
+        <x:v>0.171</x:v>
+      </x:c>
+      <x:c r="G10" s="37" t="n">
+        <x:f>0.071</x:f>
+        <x:v>0.071</x:v>
+      </x:c>
+      <x:c r="H10" s="37" t="n">
+        <x:f>PI()/4*(F10^2-G10^2)</x:f>
+        <x:v>0.019006635554218252</x:v>
+      </x:c>
+      <x:c r="I10" s="37" t="n">
+        <x:f>PI()/64*(F10^4-G10^4)</x:f>
+        <x:v>0.00004072409250435688</x:v>
+      </x:c>
+      <x:c r="J10" s="37" t="n">
+        <x:f>H10*E10*7850</x:f>
+        <x:v>13428.188019055196</x:v>
+      </x:c>
+      <x:c r="K10" s="37" t="n">
+        <x:f>0.55</x:f>
+        <x:v>0.55</x:v>
+      </x:c>
+      <x:c r="L10" s="37" t="str">
+        <x:f>"BHA component"</x:f>
+        <x:v>BHA component</x:v>
+      </x:c>
+      <x:c r="M10" s="37" t="str">
+        <x:f>IF(AND(F10&gt;G10,E10&gt;0),"PASS","REVIEW")</x:f>
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="N10" s="35"/>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" s="37" t="str">
+        <x:v>bha-hwdp-transition</x:v>
+      </x:c>
+      <x:c r="B11" s="37" t="str">
+        <x:v>HWDP transition</x:v>
+      </x:c>
+      <x:c r="C11" s="37" t="n">
+        <x:f>D10</x:f>
+        <x:v>111.8</x:v>
+      </x:c>
+      <x:c r="D11" s="37" t="n">
+        <x:f>C11+E11</x:f>
+        <x:v>171.8</x:v>
+      </x:c>
+      <x:c r="E11" s="37" t="n">
+        <x:f>60</x:f>
+        <x:v>60</x:v>
+      </x:c>
+      <x:c r="F11" s="37" t="n">
+        <x:f>0.14</x:f>
+        <x:v>0.14</x:v>
+      </x:c>
+      <x:c r="G11" s="37" t="n">
+        <x:f>0.076</x:f>
+        <x:v>0.076</x:v>
+      </x:c>
+      <x:c r="H11" s="37" t="n">
+        <x:f>PI()/4*(F11^2-G11^2)</x:f>
+        <x:v>0.010857344210806327</x:v>
+      </x:c>
+      <x:c r="I11" s="37" t="n">
+        <x:f>PI()/64*(F11^4-G11^4)</x:f>
+        <x:v>0.00001721974791833884</x:v>
+      </x:c>
+      <x:c r="J11" s="37" t="n">
+        <x:f>H11*E11*7850</x:f>
+        <x:v>5113.80912328978</x:v>
+      </x:c>
+      <x:c r="K11" s="37" t="n">
+        <x:f>0.4</x:f>
+        <x:v>0.4</x:v>
+      </x:c>
+      <x:c r="L11" s="37" t="str">
+        <x:f>"BHA component"</x:f>
+        <x:v>BHA component</x:v>
+      </x:c>
+      <x:c r="M11" s="37" t="str">
+        <x:f>IF(AND(F11&gt;G11,E11&gt;0),"PASS","REVIEW")</x:f>
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="N11" s="35"/>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A1:N1"/>
+    <x:mergeCell ref="A3:M3"/>
+  </x:mergeCells>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
@@ -7358,7 +7840,7 @@
 </x:worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
@@ -7443,7 +7925,9 @@
       <x:c r="J3" s="38" t="str">
         <x:v>Display-unit control — calculations and stored inputs remain SI</x:v>
       </x:c>
-      <x:c r="K3" s="35"/>
+      <x:c r="K3" s="38" t="str">
+        <x:v>Display-unit control — calculations and stored inputs remain SI</x:v>
+      </x:c>
       <x:c r="L3" s="35"/>
       <x:c r="M3" s="35"/>
       <x:c r="N3" s="35"/>
@@ -7481,7 +7965,7 @@
       <x:c r="H5" s="40"/>
       <x:c r="I5" s="40"/>
       <x:c r="J5" s="40"/>
-      <x:c r="K5" s="35"/>
+      <x:c r="K5" s="40"/>
       <x:c r="L5" s="35"/>
       <x:c r="M5" s="35"/>
       <x:c r="N5" s="35"/>
@@ -7533,7 +8017,9 @@
       <x:c r="J7" s="36" t="str">
         <x:v>Custom selection</x:v>
       </x:c>
-      <x:c r="K7" s="35"/>
+      <x:c r="K7" s="36" t="str">
+        <x:v>SI factor</x:v>
+      </x:c>
       <x:c r="L7" s="35"/>
       <x:c r="M7" s="35"/>
       <x:c r="N7" s="35"/>
@@ -7565,13 +8051,15 @@
         <x:v>m</x:v>
       </x:c>
       <x:c r="I8" s="18" t="n">
-        <x:f>IF($B$5="SI",1,IF($B$5="Imperial",E8,IF($B$5="Mixed",F8,IF($B$5="Custom",IF(J8="SI",1,IF(J8="Imperial",E8,IF(J8="Mixed",F8,NA()))),NA()))))</x:f>
+        <x:f>IF($B$5="SI",K8,IF($B$5="Imperial",E8,IF($B$5="Mixed",F8,IF($B$5="Custom",IF(J8="SI",K8,IF(J8="Imperial",E8,IF(J8="Mixed",F8,NA()))),NA()))))</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="J8" s="39" t="str">
         <x:v>SI</x:v>
       </x:c>
-      <x:c r="K8" s="35"/>
+      <x:c r="K8" s="41" t="n">
+        <x:v>1</x:v>
+      </x:c>
       <x:c r="L8" s="35"/>
       <x:c r="M8" s="35"/>
       <x:c r="N8" s="35"/>
@@ -7603,13 +8091,15 @@
         <x:v>m</x:v>
       </x:c>
       <x:c r="I9" s="18" t="n">
-        <x:f>IF($B$5="SI",1,IF($B$5="Imperial",E9,IF($B$5="Mixed",F9,IF($B$5="Custom",IF(J9="SI",1,IF(J9="Imperial",E9,IF(J9="Mixed",F9,NA()))),NA()))))</x:f>
+        <x:f>IF($B$5="SI",K9,IF($B$5="Imperial",E9,IF($B$5="Mixed",F9,IF($B$5="Custom",IF(J9="SI",K9,IF(J9="Imperial",E9,IF(J9="Mixed",F9,NA()))),NA()))))</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="J9" s="39" t="str">
         <x:v>SI</x:v>
       </x:c>
-      <x:c r="K9" s="35"/>
+      <x:c r="K9" s="41" t="n">
+        <x:v>1</x:v>
+      </x:c>
       <x:c r="L9" s="35"/>
       <x:c r="M9" s="35"/>
       <x:c r="N9" s="35"/>
@@ -7641,13 +8131,15 @@
         <x:v>m2</x:v>
       </x:c>
       <x:c r="I10" s="18" t="n">
-        <x:f>IF($B$5="SI",1,IF($B$5="Imperial",E10,IF($B$5="Mixed",F10,IF($B$5="Custom",IF(J10="SI",1,IF(J10="Imperial",E10,IF(J10="Mixed",F10,NA()))),NA()))))</x:f>
+        <x:f>IF($B$5="SI",K10,IF($B$5="Imperial",E10,IF($B$5="Mixed",F10,IF($B$5="Custom",IF(J10="SI",K10,IF(J10="Imperial",E10,IF(J10="Mixed",F10,NA()))),NA()))))</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="J10" s="39" t="str">
         <x:v>SI</x:v>
       </x:c>
-      <x:c r="K10" s="35"/>
+      <x:c r="K10" s="41" t="n">
+        <x:v>1</x:v>
+      </x:c>
       <x:c r="L10" s="35"/>
       <x:c r="M10" s="35"/>
       <x:c r="N10" s="35"/>
@@ -7679,13 +8171,15 @@
         <x:v>m3</x:v>
       </x:c>
       <x:c r="I11" s="18" t="n">
-        <x:f>IF($B$5="SI",1,IF($B$5="Imperial",E11,IF($B$5="Mixed",F11,IF($B$5="Custom",IF(J11="SI",1,IF(J11="Imperial",E11,IF(J11="Mixed",F11,NA()))),NA()))))</x:f>
+        <x:f>IF($B$5="SI",K11,IF($B$5="Imperial",E11,IF($B$5="Mixed",F11,IF($B$5="Custom",IF(J11="SI",K11,IF(J11="Imperial",E11,IF(J11="Mixed",F11,NA()))),NA()))))</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="J11" s="39" t="str">
         <x:v>SI</x:v>
       </x:c>
-      <x:c r="K11" s="35"/>
+      <x:c r="K11" s="41" t="n">
+        <x:v>1</x:v>
+      </x:c>
       <x:c r="L11" s="35"/>
       <x:c r="M11" s="35"/>
       <x:c r="N11" s="35"/>
@@ -7717,13 +8211,15 @@
         <x:v>m3/s</x:v>
       </x:c>
       <x:c r="I12" s="18" t="n">
-        <x:f>IF($B$5="SI",1,IF($B$5="Imperial",E12,IF($B$5="Mixed",F12,IF($B$5="Custom",IF(J12="SI",1,IF(J12="Imperial",E12,IF(J12="Mixed",F12,NA()))),NA()))))</x:f>
+        <x:f>IF($B$5="SI",K12,IF($B$5="Imperial",E12,IF($B$5="Mixed",F12,IF($B$5="Custom",IF(J12="SI",K12,IF(J12="Imperial",E12,IF(J12="Mixed",F12,NA()))),NA()))))</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="J12" s="39" t="str">
         <x:v>SI</x:v>
       </x:c>
-      <x:c r="K12" s="35"/>
+      <x:c r="K12" s="41" t="n">
+        <x:v>1</x:v>
+      </x:c>
       <x:c r="L12" s="35"/>
       <x:c r="M12" s="35"/>
       <x:c r="N12" s="35"/>
@@ -7733,35 +8229,37 @@
         <x:v>Density</x:v>
       </x:c>
       <x:c r="B13" s="41" t="str">
-        <x:v>kg/m3</x:v>
+        <x:v>g/cm3</x:v>
       </x:c>
       <x:c r="C13" s="41" t="str">
         <x:v>ppg</x:v>
       </x:c>
       <x:c r="D13" s="41" t="str">
-        <x:v>kg/m3</x:v>
+        <x:v>g/cm3</x:v>
       </x:c>
       <x:c r="E13" s="18" t="n">
         <x:v>0.008345404</x:v>
       </x:c>
       <x:c r="F13" s="18" t="n">
-        <x:v>1</x:v>
+        <x:v>0.001</x:v>
       </x:c>
       <x:c r="G13" s="18" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="H13" s="41" t="str">
         <x:f>IF($B$5="SI",B13,IF($B$5="Imperial",C13,IF($B$5="Mixed",D13,IF($B$5="Custom",IF(J13="SI",B13,IF(J13="Imperial",C13,IF(J13="Mixed",D13,"INVALID"))),"INVALID"))))</x:f>
-        <x:v>kg/m3</x:v>
+        <x:v>g/cm3</x:v>
       </x:c>
       <x:c r="I13" s="18" t="n">
-        <x:f>IF($B$5="SI",1,IF($B$5="Imperial",E13,IF($B$5="Mixed",F13,IF($B$5="Custom",IF(J13="SI",1,IF(J13="Imperial",E13,IF(J13="Mixed",F13,NA()))),NA()))))</x:f>
-        <x:v>1</x:v>
+        <x:f>IF($B$5="SI",K13,IF($B$5="Imperial",E13,IF($B$5="Mixed",F13,IF($B$5="Custom",IF(J13="SI",K13,IF(J13="Imperial",E13,IF(J13="Mixed",F13,NA()))),NA()))))</x:f>
+        <x:v>0.001</x:v>
       </x:c>
       <x:c r="J13" s="39" t="str">
         <x:v>SI</x:v>
       </x:c>
-      <x:c r="K13" s="35"/>
+      <x:c r="K13" s="41" t="n">
+        <x:v>0.001</x:v>
+      </x:c>
       <x:c r="L13" s="35"/>
       <x:c r="M13" s="35"/>
       <x:c r="N13" s="35"/>
@@ -7793,13 +8291,15 @@
         <x:v>N</x:v>
       </x:c>
       <x:c r="I14" s="18" t="n">
-        <x:f>IF($B$5="SI",1,IF($B$5="Imperial",E14,IF($B$5="Mixed",F14,IF($B$5="Custom",IF(J14="SI",1,IF(J14="Imperial",E14,IF(J14="Mixed",F14,NA()))),NA()))))</x:f>
+        <x:f>IF($B$5="SI",K14,IF($B$5="Imperial",E14,IF($B$5="Mixed",F14,IF($B$5="Custom",IF(J14="SI",K14,IF(J14="Imperial",E14,IF(J14="Mixed",F14,NA()))),NA()))))</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="J14" s="39" t="str">
         <x:v>SI</x:v>
       </x:c>
-      <x:c r="K14" s="35"/>
+      <x:c r="K14" s="41" t="n">
+        <x:v>1</x:v>
+      </x:c>
       <x:c r="L14" s="35"/>
       <x:c r="M14" s="35"/>
       <x:c r="N14" s="35"/>
@@ -7831,13 +8331,15 @@
         <x:v>Pa</x:v>
       </x:c>
       <x:c r="I15" s="18" t="n">
-        <x:f>IF($B$5="SI",1,IF($B$5="Imperial",E15,IF($B$5="Mixed",F15,IF($B$5="Custom",IF(J15="SI",1,IF(J15="Imperial",E15,IF(J15="Mixed",F15,NA()))),NA()))))</x:f>
+        <x:f>IF($B$5="SI",K15,IF($B$5="Imperial",E15,IF($B$5="Mixed",F15,IF($B$5="Custom",IF(J15="SI",K15,IF(J15="Imperial",E15,IF(J15="Mixed",F15,NA()))),NA()))))</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="J15" s="39" t="str">
         <x:v>SI</x:v>
       </x:c>
-      <x:c r="K15" s="35"/>
+      <x:c r="K15" s="41" t="n">
+        <x:v>1</x:v>
+      </x:c>
       <x:c r="L15" s="35"/>
       <x:c r="M15" s="35"/>
       <x:c r="N15" s="35"/>
@@ -7869,13 +8371,15 @@
         <x:v>N-m</x:v>
       </x:c>
       <x:c r="I16" s="18" t="n">
-        <x:f>IF($B$5="SI",1,IF($B$5="Imperial",E16,IF($B$5="Mixed",F16,IF($B$5="Custom",IF(J16="SI",1,IF(J16="Imperial",E16,IF(J16="Mixed",F16,NA()))),NA()))))</x:f>
+        <x:f>IF($B$5="SI",K16,IF($B$5="Imperial",E16,IF($B$5="Mixed",F16,IF($B$5="Custom",IF(J16="SI",K16,IF(J16="Imperial",E16,IF(J16="Mixed",F16,NA()))),NA()))))</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="J16" s="39" t="str">
         <x:v>SI</x:v>
       </x:c>
-      <x:c r="K16" s="35"/>
+      <x:c r="K16" s="41" t="n">
+        <x:v>1</x:v>
+      </x:c>
       <x:c r="L16" s="35"/>
       <x:c r="M16" s="35"/>
       <x:c r="N16" s="35"/>
@@ -7907,13 +8411,15 @@
         <x:v>Pa</x:v>
       </x:c>
       <x:c r="I17" s="18" t="n">
-        <x:f>IF($B$5="SI",1,IF($B$5="Imperial",E17,IF($B$5="Mixed",F17,IF($B$5="Custom",IF(J17="SI",1,IF(J17="Imperial",E17,IF(J17="Mixed",F17,NA()))),NA()))))</x:f>
+        <x:f>IF($B$5="SI",K17,IF($B$5="Imperial",E17,IF($B$5="Mixed",F17,IF($B$5="Custom",IF(J17="SI",K17,IF(J17="Imperial",E17,IF(J17="Mixed",F17,NA()))),NA()))))</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="J17" s="39" t="str">
         <x:v>SI</x:v>
       </x:c>
-      <x:c r="K17" s="35"/>
+      <x:c r="K17" s="41" t="n">
+        <x:v>1</x:v>
+      </x:c>
       <x:c r="L17" s="35"/>
       <x:c r="M17" s="35"/>
       <x:c r="N17" s="35"/>
@@ -7945,13 +8451,15 @@
         <x:v>rad</x:v>
       </x:c>
       <x:c r="I18" s="18" t="n">
-        <x:f>IF($B$5="SI",1,IF($B$5="Imperial",E18,IF($B$5="Mixed",F18,IF($B$5="Custom",IF(J18="SI",1,IF(J18="Imperial",E18,IF(J18="Mixed",F18,NA()))),NA()))))</x:f>
+        <x:f>IF($B$5="SI",K18,IF($B$5="Imperial",E18,IF($B$5="Mixed",F18,IF($B$5="Custom",IF(J18="SI",K18,IF(J18="Imperial",E18,IF(J18="Mixed",F18,NA()))),NA()))))</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="J18" s="39" t="str">
         <x:v>SI</x:v>
       </x:c>
-      <x:c r="K18" s="35"/>
+      <x:c r="K18" s="41" t="n">
+        <x:v>1</x:v>
+      </x:c>
       <x:c r="L18" s="35"/>
       <x:c r="M18" s="35"/>
       <x:c r="N18" s="35"/>
@@ -7983,13 +8491,15 @@
         <x:v>m/s</x:v>
       </x:c>
       <x:c r="I19" s="18" t="n">
-        <x:f>IF($B$5="SI",1,IF($B$5="Imperial",E19,IF($B$5="Mixed",F19,IF($B$5="Custom",IF(J19="SI",1,IF(J19="Imperial",E19,IF(J19="Mixed",F19,NA()))),NA()))))</x:f>
+        <x:f>IF($B$5="SI",K19,IF($B$5="Imperial",E19,IF($B$5="Mixed",F19,IF($B$5="Custom",IF(J19="SI",K19,IF(J19="Imperial",E19,IF(J19="Mixed",F19,NA()))),NA()))))</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="J19" s="39" t="str">
         <x:v>SI</x:v>
       </x:c>
-      <x:c r="K19" s="35"/>
+      <x:c r="K19" s="41" t="n">
+        <x:v>1</x:v>
+      </x:c>
       <x:c r="L19" s="35"/>
       <x:c r="M19" s="35"/>
       <x:c r="N19" s="35"/>
@@ -8021,13 +8531,15 @@
         <x:v>rad/m</x:v>
       </x:c>
       <x:c r="I20" s="18" t="n">
-        <x:f>IF($B$5="SI",1,IF($B$5="Imperial",E20,IF($B$5="Mixed",F20,IF($B$5="Custom",IF(J20="SI",1,IF(J20="Imperial",E20,IF(J20="Mixed",F20,NA()))),NA()))))</x:f>
+        <x:f>IF($B$5="SI",K20,IF($B$5="Imperial",E20,IF($B$5="Mixed",F20,IF($B$5="Custom",IF(J20="SI",K20,IF(J20="Imperial",E20,IF(J20="Mixed",F20,NA()))),NA()))))</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="J20" s="39" t="str">
         <x:v>SI</x:v>
       </x:c>
-      <x:c r="K20" s="35"/>
+      <x:c r="K20" s="41" t="n">
+        <x:v>1</x:v>
+      </x:c>
       <x:c r="L20" s="35"/>
       <x:c r="M20" s="35"/>
       <x:c r="N20" s="35"/>
@@ -8035,8 +8547,8 @@
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:N1"/>
-    <x:mergeCell ref="A3:J3"/>
-    <x:mergeCell ref="D5:J5"/>
+    <x:mergeCell ref="A3:K3"/>
+    <x:mergeCell ref="D5:K5"/>
   </x:mergeCells>
   <x:dataValidations count="14">
     <x:dataValidation type="list" sqref="B5">
@@ -8086,7 +8598,7 @@
 </x:worksheet>
 </file>
 
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
@@ -8333,7 +8845,7 @@
 </x:worksheet>
 </file>
 
-<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
@@ -9013,7 +9525,7 @@
 </x:worksheet>
 </file>
 
-<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
@@ -10656,7 +11168,7 @@
 </x:worksheet>
 </file>
 
-<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
@@ -10787,179 +11299,6 @@
   <x:mergeCells>
     <x:mergeCell ref="A1:N1"/>
     <x:mergeCell ref="A3:F3"/>
-  </x:mergeCells>
-  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</x:worksheet>
-</file>
-
-<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
-<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:sheetFormatPr defaultRowHeight="15"/>
-  <x:cols>
-    <x:col min="1" max="1" width="18" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="72" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="12" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="12" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="12" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="12" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="12" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="12" hidden="0" customWidth="1"/>
-    <x:col min="9" max="9" width="12" hidden="0" customWidth="1"/>
-    <x:col min="10" max="10" width="12" hidden="0" customWidth="1"/>
-    <x:col min="11" max="11" width="12" hidden="0" customWidth="1"/>
-    <x:col min="12" max="12" width="12" hidden="0" customWidth="1"/>
-    <x:col min="13" max="13" width="12" hidden="0" customWidth="1"/>
-    <x:col min="14" max="14" width="12" hidden="0" customWidth="1"/>
-  </x:cols>
-  <x:sheetData>
-    <x:row r="1" ht="26" customHeight="1">
-      <x:c r="A1" s="34" t="str">
-        <x:v>WellForge | Exchange Buffer | Formula-driven planning and review workbook</x:v>
-      </x:c>
-      <x:c r="B1" s="34"/>
-      <x:c r="C1" s="34"/>
-      <x:c r="D1" s="34"/>
-      <x:c r="E1" s="34"/>
-      <x:c r="F1" s="34"/>
-      <x:c r="G1" s="34"/>
-      <x:c r="H1" s="34"/>
-      <x:c r="I1" s="34"/>
-      <x:c r="J1" s="34"/>
-      <x:c r="K1" s="34"/>
-      <x:c r="L1" s="34"/>
-      <x:c r="M1" s="34"/>
-      <x:c r="N1" s="34"/>
-    </x:row>
-    <x:row r="2">
-      <x:c r="A2" s="35"/>
-      <x:c r="B2" s="35"/>
-      <x:c r="C2" s="35"/>
-      <x:c r="D2" s="35"/>
-      <x:c r="E2" s="35"/>
-      <x:c r="F2" s="35"/>
-      <x:c r="G2" s="35"/>
-      <x:c r="H2" s="35"/>
-      <x:c r="I2" s="35"/>
-      <x:c r="J2" s="35"/>
-      <x:c r="K2" s="35"/>
-      <x:c r="L2" s="35"/>
-      <x:c r="M2" s="35"/>
-      <x:c r="N2" s="35"/>
-    </x:row>
-    <x:row r="3">
-      <x:c r="A3" s="38" t="str">
-        <x:v>Office Script and desktop JSON exchange buffer</x:v>
-      </x:c>
-      <x:c r="B3" s="38" t="str">
-        <x:v>Office Script and desktop JSON exchange buffer</x:v>
-      </x:c>
-      <x:c r="C3" s="35"/>
-      <x:c r="D3" s="35"/>
-      <x:c r="E3" s="35"/>
-      <x:c r="F3" s="35"/>
-      <x:c r="G3" s="35"/>
-      <x:c r="H3" s="35"/>
-      <x:c r="I3" s="35"/>
-      <x:c r="J3" s="35"/>
-      <x:c r="K3" s="35"/>
-      <x:c r="L3" s="35"/>
-      <x:c r="M3" s="35"/>
-      <x:c r="N3" s="35"/>
-    </x:row>
-    <x:row r="4">
-      <x:c r="A4" s="35"/>
-      <x:c r="B4" s="35"/>
-      <x:c r="C4" s="35"/>
-      <x:c r="D4" s="35"/>
-      <x:c r="E4" s="35"/>
-      <x:c r="F4" s="35"/>
-      <x:c r="G4" s="35"/>
-      <x:c r="H4" s="35"/>
-      <x:c r="I4" s="35"/>
-      <x:c r="J4" s="35"/>
-      <x:c r="K4" s="35"/>
-      <x:c r="L4" s="35"/>
-      <x:c r="M4" s="35"/>
-      <x:c r="N4" s="35"/>
-    </x:row>
-    <x:row r="5" ht="96" customHeight="1">
-      <x:c r="A5" s="43" t="str">
-        <x:v>Payload</x:v>
-      </x:c>
-      <x:c r="B5" s="45" t="str"/>
-      <x:c r="C5" s="35"/>
-      <x:c r="D5" s="35"/>
-      <x:c r="E5" s="35"/>
-      <x:c r="F5" s="35"/>
-      <x:c r="G5" s="35"/>
-      <x:c r="H5" s="35"/>
-      <x:c r="I5" s="35"/>
-      <x:c r="J5" s="35"/>
-      <x:c r="K5" s="35"/>
-      <x:c r="L5" s="35"/>
-      <x:c r="M5" s="35"/>
-      <x:c r="N5" s="35"/>
-    </x:row>
-    <x:row r="6">
-      <x:c r="A6" s="43" t="str">
-        <x:v>Action</x:v>
-      </x:c>
-      <x:c r="B6" s="46" t="str"/>
-      <x:c r="C6" s="35"/>
-      <x:c r="D6" s="35"/>
-      <x:c r="E6" s="35"/>
-      <x:c r="F6" s="35"/>
-      <x:c r="G6" s="35"/>
-      <x:c r="H6" s="35"/>
-      <x:c r="I6" s="35"/>
-      <x:c r="J6" s="35"/>
-      <x:c r="K6" s="35"/>
-      <x:c r="L6" s="35"/>
-      <x:c r="M6" s="35"/>
-      <x:c r="N6" s="35"/>
-    </x:row>
-    <x:row r="7">
-      <x:c r="A7" s="43" t="str">
-        <x:v>Status</x:v>
-      </x:c>
-      <x:c r="B7" s="47" t="str">
-        <x:v>Ready</x:v>
-      </x:c>
-      <x:c r="C7" s="35"/>
-      <x:c r="D7" s="35"/>
-      <x:c r="E7" s="35"/>
-      <x:c r="F7" s="35"/>
-      <x:c r="G7" s="35"/>
-      <x:c r="H7" s="35"/>
-      <x:c r="I7" s="35"/>
-      <x:c r="J7" s="35"/>
-      <x:c r="K7" s="35"/>
-      <x:c r="L7" s="35"/>
-      <x:c r="M7" s="35"/>
-      <x:c r="N7" s="35"/>
-    </x:row>
-    <x:row r="8">
-      <x:c r="A8" s="43" t="str">
-        <x:v>Diagnostics</x:v>
-      </x:c>
-      <x:c r="B8" s="48" t="str"/>
-      <x:c r="C8" s="35"/>
-      <x:c r="D8" s="35"/>
-      <x:c r="E8" s="35"/>
-      <x:c r="F8" s="35"/>
-      <x:c r="G8" s="35"/>
-      <x:c r="H8" s="35"/>
-      <x:c r="I8" s="35"/>
-      <x:c r="J8" s="35"/>
-      <x:c r="K8" s="35"/>
-      <x:c r="L8" s="35"/>
-      <x:c r="M8" s="35"/>
-      <x:c r="N8" s="35"/>
-    </x:row>
-  </x:sheetData>
-  <x:mergeCells>
-    <x:mergeCell ref="A1:N1"/>
-    <x:mergeCell ref="A3:B3"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -11515,6 +11854,179 @@
 </x:worksheet>
 </file>
 
+<file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="18" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="72" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="12" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="12" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="12" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="12" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="12" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="12" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="12" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="12" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="12" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="12" hidden="0" customWidth="1"/>
+    <x:col min="13" max="13" width="12" hidden="0" customWidth="1"/>
+    <x:col min="14" max="14" width="12" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="26" customHeight="1">
+      <x:c r="A1" s="34" t="str">
+        <x:v>WellForge | Exchange Buffer | Formula-driven planning and review workbook</x:v>
+      </x:c>
+      <x:c r="B1" s="34"/>
+      <x:c r="C1" s="34"/>
+      <x:c r="D1" s="34"/>
+      <x:c r="E1" s="34"/>
+      <x:c r="F1" s="34"/>
+      <x:c r="G1" s="34"/>
+      <x:c r="H1" s="34"/>
+      <x:c r="I1" s="34"/>
+      <x:c r="J1" s="34"/>
+      <x:c r="K1" s="34"/>
+      <x:c r="L1" s="34"/>
+      <x:c r="M1" s="34"/>
+      <x:c r="N1" s="34"/>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" s="35"/>
+      <x:c r="B2" s="35"/>
+      <x:c r="C2" s="35"/>
+      <x:c r="D2" s="35"/>
+      <x:c r="E2" s="35"/>
+      <x:c r="F2" s="35"/>
+      <x:c r="G2" s="35"/>
+      <x:c r="H2" s="35"/>
+      <x:c r="I2" s="35"/>
+      <x:c r="J2" s="35"/>
+      <x:c r="K2" s="35"/>
+      <x:c r="L2" s="35"/>
+      <x:c r="M2" s="35"/>
+      <x:c r="N2" s="35"/>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" s="38" t="str">
+        <x:v>Office Script and desktop JSON exchange buffer</x:v>
+      </x:c>
+      <x:c r="B3" s="38" t="str">
+        <x:v>Office Script and desktop JSON exchange buffer</x:v>
+      </x:c>
+      <x:c r="C3" s="35"/>
+      <x:c r="D3" s="35"/>
+      <x:c r="E3" s="35"/>
+      <x:c r="F3" s="35"/>
+      <x:c r="G3" s="35"/>
+      <x:c r="H3" s="35"/>
+      <x:c r="I3" s="35"/>
+      <x:c r="J3" s="35"/>
+      <x:c r="K3" s="35"/>
+      <x:c r="L3" s="35"/>
+      <x:c r="M3" s="35"/>
+      <x:c r="N3" s="35"/>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" s="35"/>
+      <x:c r="B4" s="35"/>
+      <x:c r="C4" s="35"/>
+      <x:c r="D4" s="35"/>
+      <x:c r="E4" s="35"/>
+      <x:c r="F4" s="35"/>
+      <x:c r="G4" s="35"/>
+      <x:c r="H4" s="35"/>
+      <x:c r="I4" s="35"/>
+      <x:c r="J4" s="35"/>
+      <x:c r="K4" s="35"/>
+      <x:c r="L4" s="35"/>
+      <x:c r="M4" s="35"/>
+      <x:c r="N4" s="35"/>
+    </x:row>
+    <x:row r="5" ht="96" customHeight="1">
+      <x:c r="A5" s="43" t="str">
+        <x:v>Payload</x:v>
+      </x:c>
+      <x:c r="B5" s="45" t="str"/>
+      <x:c r="C5" s="35"/>
+      <x:c r="D5" s="35"/>
+      <x:c r="E5" s="35"/>
+      <x:c r="F5" s="35"/>
+      <x:c r="G5" s="35"/>
+      <x:c r="H5" s="35"/>
+      <x:c r="I5" s="35"/>
+      <x:c r="J5" s="35"/>
+      <x:c r="K5" s="35"/>
+      <x:c r="L5" s="35"/>
+      <x:c r="M5" s="35"/>
+      <x:c r="N5" s="35"/>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" s="43" t="str">
+        <x:v>Action</x:v>
+      </x:c>
+      <x:c r="B6" s="46" t="str"/>
+      <x:c r="C6" s="35"/>
+      <x:c r="D6" s="35"/>
+      <x:c r="E6" s="35"/>
+      <x:c r="F6" s="35"/>
+      <x:c r="G6" s="35"/>
+      <x:c r="H6" s="35"/>
+      <x:c r="I6" s="35"/>
+      <x:c r="J6" s="35"/>
+      <x:c r="K6" s="35"/>
+      <x:c r="L6" s="35"/>
+      <x:c r="M6" s="35"/>
+      <x:c r="N6" s="35"/>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" s="43" t="str">
+        <x:v>Status</x:v>
+      </x:c>
+      <x:c r="B7" s="47" t="str">
+        <x:v>Ready</x:v>
+      </x:c>
+      <x:c r="C7" s="35"/>
+      <x:c r="D7" s="35"/>
+      <x:c r="E7" s="35"/>
+      <x:c r="F7" s="35"/>
+      <x:c r="G7" s="35"/>
+      <x:c r="H7" s="35"/>
+      <x:c r="I7" s="35"/>
+      <x:c r="J7" s="35"/>
+      <x:c r="K7" s="35"/>
+      <x:c r="L7" s="35"/>
+      <x:c r="M7" s="35"/>
+      <x:c r="N7" s="35"/>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" s="43" t="str">
+        <x:v>Diagnostics</x:v>
+      </x:c>
+      <x:c r="B8" s="48" t="str"/>
+      <x:c r="C8" s="35"/>
+      <x:c r="D8" s="35"/>
+      <x:c r="E8" s="35"/>
+      <x:c r="F8" s="35"/>
+      <x:c r="G8" s="35"/>
+      <x:c r="H8" s="35"/>
+      <x:c r="I8" s="35"/>
+      <x:c r="J8" s="35"/>
+      <x:c r="K8" s="35"/>
+      <x:c r="L8" s="35"/>
+      <x:c r="M8" s="35"/>
+      <x:c r="N8" s="35"/>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A1:N1"/>
+    <x:mergeCell ref="A3:B3"/>
+  </x:mergeCells>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
@@ -11553,9 +12065,1656 @@
       <x:c r="M1" s="34"/>
       <x:c r="N1" s="34"/>
     </x:row>
+    <x:row r="2">
+      <x:c r="A2" s="35"/>
+      <x:c r="B2" s="35"/>
+      <x:c r="C2" s="35"/>
+      <x:c r="D2" s="35"/>
+      <x:c r="E2" s="35"/>
+      <x:c r="F2" s="35"/>
+      <x:c r="G2" s="35"/>
+      <x:c r="H2" s="35"/>
+      <x:c r="I2" s="35"/>
+      <x:c r="J2" s="35"/>
+      <x:c r="K2" s="35"/>
+      <x:c r="L2" s="35"/>
+      <x:c r="M2" s="35"/>
+      <x:c r="N2" s="35"/>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" s="38" t="str">
+        <x:v>Shared SI survey stations — reused by engineering models</x:v>
+      </x:c>
+      <x:c r="B3" s="38" t="str">
+        <x:v>Shared SI survey stations — reused by engineering models</x:v>
+      </x:c>
+      <x:c r="C3" s="38" t="str">
+        <x:v>Shared SI survey stations — reused by engineering models</x:v>
+      </x:c>
+      <x:c r="D3" s="38" t="str">
+        <x:v>Shared SI survey stations — reused by engineering models</x:v>
+      </x:c>
+      <x:c r="E3" s="38" t="str">
+        <x:v>Shared SI survey stations — reused by engineering models</x:v>
+      </x:c>
+      <x:c r="F3" s="38" t="str">
+        <x:v>Shared SI survey stations — reused by engineering models</x:v>
+      </x:c>
+      <x:c r="G3" s="35"/>
+      <x:c r="H3" s="35"/>
+      <x:c r="I3" s="35"/>
+      <x:c r="J3" s="35"/>
+      <x:c r="K3" s="35"/>
+      <x:c r="L3" s="35"/>
+      <x:c r="M3" s="35"/>
+      <x:c r="N3" s="35"/>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" s="35"/>
+      <x:c r="B4" s="35"/>
+      <x:c r="C4" s="35"/>
+      <x:c r="D4" s="35"/>
+      <x:c r="E4" s="35"/>
+      <x:c r="F4" s="35"/>
+      <x:c r="G4" s="35"/>
+      <x:c r="H4" s="35"/>
+      <x:c r="I4" s="35"/>
+      <x:c r="J4" s="35"/>
+      <x:c r="K4" s="35"/>
+      <x:c r="L4" s="35"/>
+      <x:c r="M4" s="35"/>
+      <x:c r="N4" s="35"/>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" s="36" t="str">
+        <x:v>MD m</x:v>
+      </x:c>
+      <x:c r="B5" s="36" t="str">
+        <x:v>Inclination rad</x:v>
+      </x:c>
+      <x:c r="C5" s="36" t="str">
+        <x:v>Azimuth rad</x:v>
+      </x:c>
+      <x:c r="D5" s="36" t="str">
+        <x:v>Hole ID m</x:v>
+      </x:c>
+      <x:c r="E5" s="36" t="str">
+        <x:v>Exchange record ID</x:v>
+      </x:c>
+      <x:c r="F5" s="35"/>
+      <x:c r="G5" s="35"/>
+      <x:c r="H5" s="35"/>
+      <x:c r="I5" s="35"/>
+      <x:c r="J5" s="35"/>
+      <x:c r="K5" s="35"/>
+      <x:c r="L5" s="35"/>
+      <x:c r="M5" s="35"/>
+      <x:c r="N5" s="35"/>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" s="39" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="B6" s="39" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C6" s="39" t="n">
+        <x:v>0.3490658503988659</x:v>
+      </x:c>
+      <x:c r="D6" s="39" t="n">
+        <x:v>0.216</x:v>
+      </x:c>
+      <x:c r="E6" s="35" t="str">
+        <x:v>survey-000</x:v>
+      </x:c>
+      <x:c r="F6" s="35"/>
+      <x:c r="G6" s="35"/>
+      <x:c r="H6" s="35"/>
+      <x:c r="I6" s="35"/>
+      <x:c r="J6" s="35"/>
+      <x:c r="K6" s="35"/>
+      <x:c r="L6" s="35"/>
+      <x:c r="M6" s="35"/>
+      <x:c r="N6" s="35"/>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" s="39" t="n">
+        <x:v>155.10875760000002</x:v>
+      </x:c>
+      <x:c r="B7" s="39" t="n">
+        <x:v>0.008499753457212385</x:v>
+      </x:c>
+      <x:c r="C7" s="39" t="n">
+        <x:v>0.36271432514946156</x:v>
+      </x:c>
+      <x:c r="D7" s="39" t="n">
+        <x:v>0.216</x:v>
+      </x:c>
+      <x:c r="E7" s="35" t="str">
+        <x:v>survey-001</x:v>
+      </x:c>
+      <x:c r="F7" s="35"/>
+      <x:c r="G7" s="35"/>
+      <x:c r="H7" s="35"/>
+      <x:c r="I7" s="35"/>
+      <x:c r="J7" s="35"/>
+      <x:c r="K7" s="35"/>
+      <x:c r="L7" s="35"/>
+      <x:c r="M7" s="35"/>
+      <x:c r="N7" s="35"/>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" s="39" t="n">
+        <x:v>307.974492</x:v>
+      </x:c>
+      <x:c r="B8" s="39" t="n">
+        <x:v>0.010454522219446033</x:v>
+      </x:c>
+      <x:c r="C8" s="39" t="n">
+        <x:v>0.36976545532751864</x:v>
+      </x:c>
+      <x:c r="D8" s="39" t="n">
+        <x:v>0.216</x:v>
+      </x:c>
+      <x:c r="E8" s="35" t="str">
+        <x:v>survey-002</x:v>
+      </x:c>
+      <x:c r="F8" s="35"/>
+      <x:c r="G8" s="35"/>
+      <x:c r="H8" s="35"/>
+      <x:c r="I8" s="35"/>
+      <x:c r="J8" s="35"/>
+      <x:c r="K8" s="35"/>
+      <x:c r="L8" s="35"/>
+      <x:c r="M8" s="35"/>
+      <x:c r="N8" s="35"/>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" s="39" t="n">
+        <x:v>460.2227016</x:v>
+      </x:c>
+      <x:c r="B9" s="39" t="n">
+        <x:v>0.007766715171374767</x:v>
+      </x:c>
+      <x:c r="C9" s="39" t="n">
+        <x:v>0.36681584889164826</x:v>
+      </x:c>
+      <x:c r="D9" s="39" t="n">
+        <x:v>0.216</x:v>
+      </x:c>
+      <x:c r="E9" s="35" t="str">
+        <x:v>survey-003</x:v>
+      </x:c>
+      <x:c r="F9" s="35"/>
+      <x:c r="G9" s="35"/>
+      <x:c r="H9" s="35"/>
+      <x:c r="I9" s="35"/>
+      <x:c r="J9" s="35"/>
+      <x:c r="K9" s="35"/>
+      <x:c r="L9" s="35"/>
+      <x:c r="M9" s="35"/>
+      <x:c r="N9" s="35"/>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" s="39" t="n">
+        <x:v>611.9649432</x:v>
+      </x:c>
+      <x:c r="B10" s="39" t="n">
+        <x:v>0.004153883619746505</x:v>
+      </x:c>
+      <x:c r="C10" s="39" t="n">
+        <x:v>0.3552792225359658</x:v>
+      </x:c>
+      <x:c r="D10" s="39" t="n">
+        <x:v>0.216</x:v>
+      </x:c>
+      <x:c r="E10" s="35" t="str">
+        <x:v>survey-004</x:v>
+      </x:c>
+      <x:c r="F10" s="35"/>
+      <x:c r="G10" s="35"/>
+      <x:c r="H10" s="35"/>
+      <x:c r="I10" s="35"/>
+      <x:c r="J10" s="35"/>
+      <x:c r="K10" s="35"/>
+      <x:c r="L10" s="35"/>
+      <x:c r="M10" s="35"/>
+      <x:c r="N10" s="35"/>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" s="39" t="n">
+        <x:v>763.5706344</x:v>
+      </x:c>
+      <x:c r="B11" s="39" t="n">
+        <x:v>0.009145525280450286</x:v>
+      </x:c>
+      <x:c r="C11" s="39" t="n">
+        <x:v>0.34074062986685294</x:v>
+      </x:c>
+      <x:c r="D11" s="39" t="n">
+        <x:v>0.216</x:v>
+      </x:c>
+      <x:c r="E11" s="35" t="str">
+        <x:v>survey-005</x:v>
+      </x:c>
+      <x:c r="F11" s="35"/>
+      <x:c r="G11" s="35"/>
+      <x:c r="H11" s="35"/>
+      <x:c r="I11" s="35"/>
+      <x:c r="J11" s="35"/>
+      <x:c r="K11" s="35"/>
+      <x:c r="L11" s="35"/>
+      <x:c r="M11" s="35"/>
+      <x:c r="N11" s="35"/>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" s="39" t="n">
+        <x:v>915.4786872000001</x:v>
+      </x:c>
+      <x:c r="B12" s="39" t="n">
+        <x:v>0.010314895879286487</x:v>
+      </x:c>
+      <x:c r="C12" s="39" t="n">
+        <x:v>0.3302337477698471</x:v>
+      </x:c>
+      <x:c r="D12" s="39" t="n">
+        <x:v>0.216</x:v>
+      </x:c>
+      <x:c r="E12" s="35" t="str">
+        <x:v>survey-006</x:v>
+      </x:c>
+      <x:c r="F12" s="35"/>
+      <x:c r="G12" s="35"/>
+      <x:c r="H12" s="35"/>
+      <x:c r="I12" s="35"/>
+      <x:c r="J12" s="35"/>
+      <x:c r="K12" s="35"/>
+      <x:c r="L12" s="35"/>
+      <x:c r="M12" s="35"/>
+      <x:c r="N12" s="35"/>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" s="39" t="n">
+        <x:v>1067.9740896</x:v>
+      </x:c>
+      <x:c r="B13" s="39" t="n">
+        <x:v>0.006928957130417489</x:v>
+      </x:c>
+      <x:c r="C13" s="39" t="n">
+        <x:v>0.32882003107573166</x:v>
+      </x:c>
+      <x:c r="D13" s="39" t="n">
+        <x:v>0.216</x:v>
+      </x:c>
+      <x:c r="E13" s="35" t="str">
+        <x:v>survey-007</x:v>
+      </x:c>
+      <x:c r="F13" s="35"/>
+      <x:c r="G13" s="35"/>
+      <x:c r="H13" s="35"/>
+      <x:c r="I13" s="35"/>
+      <x:c r="J13" s="35"/>
+      <x:c r="K13" s="35"/>
+      <x:c r="L13" s="35"/>
+      <x:c r="M13" s="35"/>
+      <x:c r="N13" s="35"/>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" s="39" t="n">
+        <x:v>1221.042516</x:v>
+      </x:c>
+      <x:c r="B14" s="39" t="n">
+        <x:v>0.005148721293383272</x:v>
+      </x:c>
+      <x:c r="C14" s="39" t="n">
+        <x:v>0.3371801581927845</x:v>
+      </x:c>
+      <x:c r="D14" s="39" t="n">
+        <x:v>0.216</x:v>
+      </x:c>
+      <x:c r="E14" s="35" t="str">
+        <x:v>survey-008</x:v>
+      </x:c>
+      <x:c r="F14" s="35"/>
+      <x:c r="G14" s="35"/>
+      <x:c r="H14" s="35"/>
+      <x:c r="I14" s="35"/>
+      <x:c r="J14" s="35"/>
+      <x:c r="K14" s="35"/>
+      <x:c r="L14" s="35"/>
+      <x:c r="M14" s="35"/>
+      <x:c r="N14" s="35"/>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" s="39" t="n">
+        <x:v>1374.3773376000001</x:v>
+      </x:c>
+      <x:c r="B15" s="39" t="n">
+        <x:v>0.009669124056048585</x:v>
+      </x:c>
+      <x:c r="C15" s="39" t="n">
+        <x:v>0.35129987184141864</x:v>
+      </x:c>
+      <x:c r="D15" s="39" t="n">
+        <x:v>0.216</x:v>
+      </x:c>
+      <x:c r="E15" s="35" t="str">
+        <x:v>survey-009</x:v>
+      </x:c>
+      <x:c r="F15" s="35"/>
+      <x:c r="G15" s="35"/>
+      <x:c r="H15" s="35"/>
+      <x:c r="I15" s="35"/>
+      <x:c r="J15" s="35"/>
+      <x:c r="K15" s="35"/>
+      <x:c r="L15" s="35"/>
+      <x:c r="M15" s="35"/>
+      <x:c r="N15" s="35"/>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" s="39" t="n">
+        <x:v>1527.5362896000001</x:v>
+      </x:c>
+      <x:c r="B16" s="39" t="n">
+        <x:v>0.010035643198967393</x:v>
+      </x:c>
+      <x:c r="C16" s="39" t="n">
+        <x:v>0.36433748135381633</x:v>
+      </x:c>
+      <x:c r="D16" s="39" t="n">
+        <x:v>0.216</x:v>
+      </x:c>
+      <x:c r="E16" s="35" t="str">
+        <x:v>survey-010</x:v>
+      </x:c>
+      <x:c r="F16" s="35"/>
+      <x:c r="G16" s="35"/>
+      <x:c r="H16" s="35"/>
+      <x:c r="I16" s="35"/>
+      <x:c r="J16" s="35"/>
+      <x:c r="K16" s="35"/>
+      <x:c r="L16" s="35"/>
+      <x:c r="M16" s="35"/>
+      <x:c r="N16" s="35"/>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" s="39" t="n">
+        <x:v>1565.8667184</x:v>
+      </x:c>
+      <x:c r="B17" s="39" t="n">
+        <x:v>0.20598375832037077</x:v>
+      </x:c>
+      <x:c r="C17" s="39" t="n">
+        <x:v>0.43128831146031876</x:v>
+      </x:c>
+      <x:c r="D17" s="39" t="n">
+        <x:v>0.216</x:v>
+      </x:c>
+      <x:c r="E17" s="35" t="str">
+        <x:v>survey-011</x:v>
+      </x:c>
+      <x:c r="F17" s="35"/>
+      <x:c r="G17" s="35"/>
+      <x:c r="H17" s="35"/>
+      <x:c r="I17" s="35"/>
+      <x:c r="J17" s="35"/>
+      <x:c r="K17" s="35"/>
+      <x:c r="L17" s="35"/>
+      <x:c r="M17" s="35"/>
+      <x:c r="N17" s="35"/>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" s="39" t="n">
+        <x:v>1603.5857184000001</x:v>
+      </x:c>
+      <x:c r="B18" s="39" t="n">
+        <x:v>0.38554323176554733</x:v>
+      </x:c>
+      <x:c r="C18" s="39" t="n">
+        <x:v>0.47877872040708447</x:v>
+      </x:c>
+      <x:c r="D18" s="39" t="n">
+        <x:v>0.216</x:v>
+      </x:c>
+      <x:c r="E18" s="35" t="str">
+        <x:v>survey-012</x:v>
+      </x:c>
+      <x:c r="F18" s="35"/>
+      <x:c r="G18" s="35"/>
+      <x:c r="H18" s="35"/>
+      <x:c r="I18" s="35"/>
+      <x:c r="J18" s="35"/>
+      <x:c r="K18" s="35"/>
+      <x:c r="L18" s="35"/>
+      <x:c r="M18" s="35"/>
+      <x:c r="N18" s="35"/>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19" s="39" t="n">
+        <x:v>1640.9209752000002</x:v>
+      </x:c>
+      <x:c r="B19" s="39" t="n">
+        <x:v>0.5509829915620899</x:v>
+      </x:c>
+      <x:c r="C19" s="39" t="n">
+        <x:v>0.5133711461816121</x:v>
+      </x:c>
+      <x:c r="D19" s="39" t="n">
+        <x:v>0.216</x:v>
+      </x:c>
+      <x:c r="E19" s="35" t="str">
+        <x:v>survey-013</x:v>
+      </x:c>
+      <x:c r="F19" s="35"/>
+      <x:c r="G19" s="35"/>
+      <x:c r="H19" s="35"/>
+      <x:c r="I19" s="35"/>
+      <x:c r="J19" s="35"/>
+      <x:c r="K19" s="35"/>
+      <x:c r="L19" s="35"/>
+      <x:c r="M19" s="35"/>
+      <x:c r="N19" s="35"/>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" s="39" t="n">
+        <x:v>1678.2970752</x:v>
+      </x:c>
+      <x:c r="B20" s="39" t="n">
+        <x:v>0.7084815032620583</x:v>
+      </x:c>
+      <x:c r="C20" s="39" t="n">
+        <x:v>0.5371599838862948</x:v>
+      </x:c>
+      <x:c r="D20" s="39" t="n">
+        <x:v>0.216</x:v>
+      </x:c>
+      <x:c r="E20" s="35" t="str">
+        <x:v>survey-014</x:v>
+      </x:c>
+      <x:c r="F20" s="35"/>
+      <x:c r="G20" s="35"/>
+      <x:c r="H20" s="35"/>
+      <x:c r="I20" s="35"/>
+      <x:c r="J20" s="35"/>
+      <x:c r="K20" s="35"/>
+      <x:c r="L20" s="35"/>
+      <x:c r="M20" s="35"/>
+      <x:c r="N20" s="35"/>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21" s="39" t="n">
+        <x:v>1716.1166592000002</x:v>
+      </x:c>
+      <x:c r="B21" s="39" t="n">
+        <x:v>0.8696277530986946</x:v>
+      </x:c>
+      <x:c r="C21" s="39" t="n">
+        <x:v>0.5575803361346284</x:v>
+      </x:c>
+      <x:c r="D21" s="39" t="n">
+        <x:v>0.216</x:v>
+      </x:c>
+      <x:c r="E21" s="35" t="str">
+        <x:v>survey-015</x:v>
+      </x:c>
+      <x:c r="F21" s="35"/>
+      <x:c r="G21" s="35"/>
+      <x:c r="H21" s="35"/>
+      <x:c r="I21" s="35"/>
+      <x:c r="J21" s="35"/>
+      <x:c r="K21" s="35"/>
+      <x:c r="L21" s="35"/>
+      <x:c r="M21" s="35"/>
+      <x:c r="N21" s="35"/>
+    </x:row>
+    <x:row r="22">
+      <x:c r="A22" s="39" t="n">
+        <x:v>1754.5571208000001</x:v>
+      </x:c>
+      <x:c r="B22" s="39" t="n">
+        <x:v>1.0435149064748896</x:v>
+      </x:c>
+      <x:c r="C22" s="39" t="n">
+        <x:v>0.5837602749145435</x:v>
+      </x:c>
+      <x:c r="D22" s="39" t="n">
+        <x:v>0.216</x:v>
+      </x:c>
+      <x:c r="E22" s="35" t="str">
+        <x:v>survey-016</x:v>
+      </x:c>
+      <x:c r="F22" s="35"/>
+      <x:c r="G22" s="35"/>
+      <x:c r="H22" s="35"/>
+      <x:c r="I22" s="35"/>
+      <x:c r="J22" s="35"/>
+      <x:c r="K22" s="35"/>
+      <x:c r="L22" s="35"/>
+      <x:c r="M22" s="35"/>
+      <x:c r="N22" s="35"/>
+    </x:row>
+    <x:row r="23">
+      <x:c r="A23" s="39" t="n">
+        <x:v>1793.4788616</x:v>
+      </x:c>
+      <x:c r="B23" s="39" t="n">
+        <x:v>1.2305967489961618</x:v>
+      </x:c>
+      <x:c r="C23" s="39" t="n">
+        <x:v>0.6219480789481793</x:v>
+      </x:c>
+      <x:c r="D23" s="39" t="n">
+        <x:v>0.216</x:v>
+      </x:c>
+      <x:c r="E23" s="35" t="str">
+        <x:v>survey-017</x:v>
+      </x:c>
+      <x:c r="F23" s="35"/>
+      <x:c r="G23" s="35"/>
+      <x:c r="H23" s="35"/>
+      <x:c r="I23" s="35"/>
+      <x:c r="J23" s="35"/>
+      <x:c r="K23" s="35"/>
+      <x:c r="L23" s="35"/>
+      <x:c r="M23" s="35"/>
+      <x:c r="N23" s="35"/>
+    </x:row>
+    <x:row r="24">
+      <x:c r="A24" s="39" t="n">
+        <x:v>1832.4975288000003</x:v>
+      </x:c>
+      <x:c r="B24" s="39" t="n">
+        <x:v>1.422321167327739</x:v>
+      </x:c>
+      <x:c r="C24" s="39" t="n">
+        <x:v>0.6724404542083752</x:v>
+      </x:c>
+      <x:c r="D24" s="39" t="n">
+        <x:v>0.216</x:v>
+      </x:c>
+      <x:c r="E24" s="35" t="str">
+        <x:v>survey-018</x:v>
+      </x:c>
+      <x:c r="F24" s="35"/>
+      <x:c r="G24" s="35"/>
+      <x:c r="H24" s="35"/>
+      <x:c r="I24" s="35"/>
+      <x:c r="J24" s="35"/>
+      <x:c r="K24" s="35"/>
+      <x:c r="L24" s="35"/>
+      <x:c r="M24" s="35"/>
+      <x:c r="N24" s="35"/>
+    </x:row>
+    <x:row r="25">
+      <x:c r="A25" s="39" t="n">
+        <x:v>1871.1787824</x:v>
+      </x:c>
+      <x:c r="B25" s="39" t="n">
+        <x:v>1.607011908773779</x:v>
+      </x:c>
+      <x:c r="C25" s="39" t="n">
+        <x:v>0.7294254542859901</x:v>
+      </x:c>
+      <x:c r="D25" s="39" t="n">
+        <x:v>0.216</x:v>
+      </x:c>
+      <x:c r="E25" s="35" t="str">
+        <x:v>survey-019</x:v>
+      </x:c>
+      <x:c r="F25" s="35"/>
+      <x:c r="G25" s="35"/>
+      <x:c r="H25" s="35"/>
+      <x:c r="I25" s="35"/>
+      <x:c r="J25" s="35"/>
+      <x:c r="K25" s="35"/>
+      <x:c r="L25" s="35"/>
+      <x:c r="M25" s="35"/>
+      <x:c r="N25" s="35"/>
+    </x:row>
+    <x:row r="26">
+      <x:c r="A26" s="39" t="n">
+        <x:v>1947.3607992000002</x:v>
+      </x:c>
+      <x:c r="B26" s="39" t="n">
+        <x:v>1.5600974584801712</x:v>
+      </x:c>
+      <x:c r="C26" s="39" t="n">
+        <x:v>0.775345066905961</x:v>
+      </x:c>
+      <x:c r="D26" s="39" t="n">
+        <x:v>0.216</x:v>
+      </x:c>
+      <x:c r="E26" s="35" t="str">
+        <x:v>survey-020</x:v>
+      </x:c>
+      <x:c r="F26" s="35"/>
+      <x:c r="G26" s="35"/>
+      <x:c r="H26" s="35"/>
+      <x:c r="I26" s="35"/>
+      <x:c r="J26" s="35"/>
+      <x:c r="K26" s="35"/>
+      <x:c r="L26" s="35"/>
+      <x:c r="M26" s="35"/>
+      <x:c r="N26" s="35"/>
+    </x:row>
+    <x:row r="27">
+      <x:c r="A27" s="39" t="n">
+        <x:v>2022.9868608</x:v>
+      </x:c>
+      <x:c r="B27" s="39" t="n">
+        <x:v>1.5621045871199648</x:v>
+      </x:c>
+      <x:c r="C27" s="39" t="n">
+        <x:v>0.8168664498109061</x:v>
+      </x:c>
+      <x:c r="D27" s="39" t="n">
+        <x:v>0.216</x:v>
+      </x:c>
+      <x:c r="E27" s="35" t="str">
+        <x:v>survey-021</x:v>
+      </x:c>
+      <x:c r="F27" s="35"/>
+      <x:c r="G27" s="35"/>
+      <x:c r="H27" s="35"/>
+      <x:c r="I27" s="35"/>
+      <x:c r="J27" s="35"/>
+      <x:c r="K27" s="35"/>
+      <x:c r="L27" s="35"/>
+      <x:c r="M27" s="35"/>
+      <x:c r="N27" s="35"/>
+    </x:row>
+    <x:row r="28">
+      <x:c r="A28" s="39" t="n">
+        <x:v>2098.3837128</x:v>
+      </x:c>
+      <x:c r="B28" s="39" t="n">
+        <x:v>1.5629597984534422</x:v>
+      </x:c>
+      <x:c r="C28" s="39" t="n">
+        <x:v>0.8568519429740961</x:v>
+      </x:c>
+      <x:c r="D28" s="39" t="n">
+        <x:v>0.216</x:v>
+      </x:c>
+      <x:c r="E28" s="35" t="str">
+        <x:v>survey-022</x:v>
+      </x:c>
+      <x:c r="F28" s="35"/>
+      <x:c r="G28" s="35"/>
+      <x:c r="H28" s="35"/>
+      <x:c r="I28" s="35"/>
+      <x:c r="J28" s="35"/>
+      <x:c r="K28" s="35"/>
+      <x:c r="L28" s="35"/>
+      <x:c r="M28" s="35"/>
+      <x:c r="N28" s="35"/>
+    </x:row>
+    <x:row r="29">
+      <x:c r="A29" s="39" t="n">
+        <x:v>2173.9945344000002</x:v>
+      </x:c>
+      <x:c r="B29" s="39" t="n">
+        <x:v>1.5629074385758823</x:v>
+      </x:c>
+      <x:c r="C29" s="39" t="n">
+        <x:v>0.8946034146947335</x:v>
+      </x:c>
+      <x:c r="D29" s="39" t="n">
+        <x:v>0.216</x:v>
+      </x:c>
+      <x:c r="E29" s="35" t="str">
+        <x:v>survey-023</x:v>
+      </x:c>
+      <x:c r="F29" s="35"/>
+      <x:c r="G29" s="35"/>
+      <x:c r="H29" s="35"/>
+      <x:c r="I29" s="35"/>
+      <x:c r="J29" s="35"/>
+      <x:c r="K29" s="35"/>
+      <x:c r="L29" s="35"/>
+      <x:c r="M29" s="35"/>
+      <x:c r="N29" s="35"/>
+    </x:row>
+    <x:row r="30">
+      <x:c r="A30" s="39" t="n">
+        <x:v>2250.1543008</x:v>
+      </x:c>
+      <x:c r="B30" s="39" t="n">
+        <x:v>1.5623314799227241</x:v>
+      </x:c>
+      <x:c r="C30" s="39" t="n">
+        <x:v>0.9295274530271401</x:v>
+      </x:c>
+      <x:c r="D30" s="39" t="n">
+        <x:v>0.216</x:v>
+      </x:c>
+      <x:c r="E30" s="35" t="str">
+        <x:v>survey-024</x:v>
+      </x:c>
+      <x:c r="F30" s="35"/>
+      <x:c r="G30" s="35"/>
+      <x:c r="H30" s="35"/>
+      <x:c r="I30" s="35"/>
+      <x:c r="J30" s="35"/>
+      <x:c r="K30" s="35"/>
+      <x:c r="L30" s="35"/>
+      <x:c r="M30" s="35"/>
+      <x:c r="N30" s="35"/>
+    </x:row>
+    <x:row r="31">
+      <x:c r="A31" s="39" t="n">
+        <x:v>2326.9172664000002</x:v>
+      </x:c>
+      <x:c r="B31" s="39" t="n">
+        <x:v>1.5615111751742867</x:v>
+      </x:c>
+      <x:c r="C31" s="39" t="n">
+        <x:v>0.9611528190732773</x:v>
+      </x:c>
+      <x:c r="D31" s="39" t="n">
+        <x:v>0.216</x:v>
+      </x:c>
+      <x:c r="E31" s="35" t="str">
+        <x:v>survey-025</x:v>
+      </x:c>
+      <x:c r="F31" s="35"/>
+      <x:c r="G31" s="35"/>
+      <x:c r="H31" s="35"/>
+      <x:c r="I31" s="35"/>
+      <x:c r="J31" s="35"/>
+      <x:c r="K31" s="35"/>
+      <x:c r="L31" s="35"/>
+      <x:c r="M31" s="35"/>
+      <x:c r="N31" s="35"/>
+    </x:row>
+    <x:row r="32">
+      <x:c r="A32" s="39" t="n">
+        <x:v>2404.030752</x:v>
+      </x:c>
+      <x:c r="B32" s="39" t="n">
+        <x:v>1.5605686973782098</x:v>
+      </x:c>
+      <x:c r="C32" s="39" t="n">
+        <x:v>0.9891479002752662</x:v>
+      </x:c>
+      <x:c r="D32" s="39" t="n">
+        <x:v>0.216</x:v>
+      </x:c>
+      <x:c r="E32" s="35" t="str">
+        <x:v>survey-026</x:v>
+      </x:c>
+      <x:c r="F32" s="35"/>
+      <x:c r="G32" s="35"/>
+      <x:c r="H32" s="35"/>
+      <x:c r="I32" s="35"/>
+      <x:c r="J32" s="35"/>
+      <x:c r="K32" s="35"/>
+      <x:c r="L32" s="35"/>
+      <x:c r="M32" s="35"/>
+      <x:c r="N32" s="35"/>
+    </x:row>
+    <x:row r="33">
+      <x:c r="A33" s="39" t="n">
+        <x:v>2481.0637704</x:v>
+      </x:c>
+      <x:c r="B33" s="39" t="n">
+        <x:v>1.5594516866569332</x:v>
+      </x:c>
+      <x:c r="C33" s="39" t="n">
+        <x:v>1.0132858038303478</x:v>
+      </x:c>
+      <x:c r="D33" s="39" t="n">
+        <x:v>0.216</x:v>
+      </x:c>
+      <x:c r="E33" s="35" t="str">
+        <x:v>survey-027</x:v>
+      </x:c>
+      <x:c r="F33" s="35"/>
+      <x:c r="G33" s="35"/>
+      <x:c r="H33" s="35"/>
+      <x:c r="I33" s="35"/>
+      <x:c r="J33" s="35"/>
+      <x:c r="K33" s="35"/>
+      <x:c r="L33" s="35"/>
+      <x:c r="M33" s="35"/>
+      <x:c r="N33" s="35"/>
+    </x:row>
+    <x:row r="34">
+      <x:c r="A34" s="39" t="n">
+        <x:v>2557.6252632</x:v>
+      </x:c>
+      <x:c r="B34" s="39" t="n">
+        <x:v>1.5579332502076986</x:v>
+      </x:c>
+      <x:c r="C34" s="39" t="n">
+        <x:v>1.0335665297385221</x:v>
+      </x:c>
+      <x:c r="D34" s="39" t="n">
+        <x:v>0.216</x:v>
+      </x:c>
+      <x:c r="E34" s="35" t="str">
+        <x:v>survey-028</x:v>
+      </x:c>
+      <x:c r="F34" s="35"/>
+      <x:c r="G34" s="35"/>
+      <x:c r="H34" s="35"/>
+      <x:c r="I34" s="35"/>
+      <x:c r="J34" s="35"/>
+      <x:c r="K34" s="35"/>
+      <x:c r="L34" s="35"/>
+      <x:c r="M34" s="35"/>
+      <x:c r="N34" s="35"/>
+    </x:row>
+    <x:row r="35">
+      <x:c r="A35" s="39" t="n">
+        <x:v>2633.5658784</x:v>
+      </x:c>
+      <x:c r="B35" s="39" t="n">
+        <x:v>1.5558039485202655</x:v>
+      </x:c>
+      <x:c r="C35" s="39" t="n">
+        <x:v>1.0500598911698684</x:v>
+      </x:c>
+      <x:c r="D35" s="39" t="n">
+        <x:v>0.216</x:v>
+      </x:c>
+      <x:c r="E35" s="35" t="str">
+        <x:v>survey-029</x:v>
+      </x:c>
+      <x:c r="F35" s="35"/>
+      <x:c r="G35" s="35"/>
+      <x:c r="H35" s="35"/>
+      <x:c r="I35" s="35"/>
+      <x:c r="J35" s="35"/>
+      <x:c r="K35" s="35"/>
+      <x:c r="L35" s="35"/>
+      <x:c r="M35" s="35"/>
+      <x:c r="N35" s="35"/>
+    </x:row>
+    <x:row r="36">
+      <x:c r="A36" s="39" t="n">
+        <x:v>2709.0514272</x:v>
+      </x:c>
+      <x:c r="B36" s="39" t="n">
+        <x:v>1.5529590618395142</x:v>
+      </x:c>
+      <x:c r="C36" s="39" t="n">
+        <x:v>1.0630451408047061</x:v>
+      </x:c>
+      <x:c r="D36" s="39" t="n">
+        <x:v>0.216</x:v>
+      </x:c>
+      <x:c r="E36" s="35" t="str">
+        <x:v>survey-030</x:v>
+      </x:c>
+      <x:c r="F36" s="35"/>
+      <x:c r="G36" s="35"/>
+      <x:c r="H36" s="35"/>
+      <x:c r="I36" s="35"/>
+      <x:c r="J36" s="35"/>
+      <x:c r="K36" s="35"/>
+      <x:c r="L36" s="35"/>
+      <x:c r="M36" s="35"/>
+      <x:c r="N36" s="35"/>
+    </x:row>
+    <x:row r="37">
+      <x:c r="A37" s="39" t="n">
+        <x:v>2784.480588</x:v>
+      </x:c>
+      <x:c r="B37" s="39" t="n">
+        <x:v>1.5494858566280458</x:v>
+      </x:c>
+      <x:c r="C37" s="39" t="n">
+        <x:v>1.0729062510784741</x:v>
+      </x:c>
+      <x:c r="D37" s="39" t="n">
+        <x:v>0.216</x:v>
+      </x:c>
+      <x:c r="E37" s="35" t="str">
+        <x:v>survey-031</x:v>
+      </x:c>
+      <x:c r="F37" s="35"/>
+      <x:c r="G37" s="35"/>
+      <x:c r="H37" s="35"/>
+      <x:c r="I37" s="35"/>
+      <x:c r="J37" s="35"/>
+      <x:c r="K37" s="35"/>
+      <x:c r="L37" s="35"/>
+      <x:c r="M37" s="35"/>
+      <x:c r="N37" s="35"/>
+    </x:row>
+    <x:row r="38">
+      <x:c r="A38" s="39" t="n">
+        <x:v>2860.2800807999997</x:v>
+      </x:c>
+      <x:c r="B38" s="39" t="n">
+        <x:v>1.5457333987362578</x:v>
+      </x:c>
+      <x:c r="C38" s="39" t="n">
+        <x:v>1.0801319141817307</x:v>
+      </x:c>
+      <x:c r="D38" s="39" t="n">
+        <x:v>0.216</x:v>
+      </x:c>
+      <x:c r="E38" s="35" t="str">
+        <x:v>survey-032</x:v>
+      </x:c>
+      <x:c r="F38" s="35"/>
+      <x:c r="G38" s="35"/>
+      <x:c r="H38" s="35"/>
+      <x:c r="I38" s="35"/>
+      <x:c r="J38" s="35"/>
+      <x:c r="K38" s="35"/>
+      <x:c r="L38" s="35"/>
+      <x:c r="M38" s="35"/>
+      <x:c r="N38" s="35"/>
+    </x:row>
+    <x:row r="39">
+      <x:c r="A39" s="39" t="n">
+        <x:v>2936.688564</x:v>
+      </x:c>
+      <x:c r="B39" s="39" t="n">
+        <x:v>1.5422776468173092</x:v>
+      </x:c>
+      <x:c r="C39" s="39" t="n">
+        <x:v>1.0852806354751139</x:v>
+      </x:c>
+      <x:c r="D39" s="39" t="n">
+        <x:v>0.216</x:v>
+      </x:c>
+      <x:c r="E39" s="35" t="str">
+        <x:v>survey-033</x:v>
+      </x:c>
+      <x:c r="F39" s="35"/>
+      <x:c r="G39" s="35"/>
+      <x:c r="H39" s="35"/>
+      <x:c r="I39" s="35"/>
+      <x:c r="J39" s="35"/>
+      <x:c r="K39" s="35"/>
+      <x:c r="L39" s="35"/>
+      <x:c r="M39" s="35"/>
+      <x:c r="N39" s="35"/>
+    </x:row>
+    <x:row r="40">
+      <x:c r="A40" s="39" t="n">
+        <x:v>3013.6334952</x:v>
+      </x:c>
+      <x:c r="B40" s="39" t="n">
+        <x:v>1.5397818259869571</x:v>
+      </x:c>
+      <x:c r="C40" s="39" t="n">
+        <x:v>1.0889981867818619</x:v>
+      </x:c>
+      <x:c r="D40" s="39" t="n">
+        <x:v>0.216</x:v>
+      </x:c>
+      <x:c r="E40" s="35" t="str">
+        <x:v>survey-034</x:v>
+      </x:c>
+      <x:c r="F40" s="35"/>
+      <x:c r="G40" s="35"/>
+      <x:c r="H40" s="35"/>
+      <x:c r="I40" s="35"/>
+      <x:c r="J40" s="35"/>
+      <x:c r="K40" s="35"/>
+      <x:c r="L40" s="35"/>
+      <x:c r="M40" s="35"/>
+      <x:c r="N40" s="35"/>
+    </x:row>
+    <x:row r="41">
+      <x:c r="A41" s="39" t="n">
+        <x:v>3090.7698408</x:v>
+      </x:c>
+      <x:c r="B41" s="39" t="n">
+        <x:v>1.5388917080684403</x:v>
+      </x:c>
+      <x:c r="C41" s="39" t="n">
+        <x:v>1.0919303399252125</x:v>
+      </x:c>
+      <x:c r="D41" s="39" t="n">
+        <x:v>0.216</x:v>
+      </x:c>
+      <x:c r="E41" s="35" t="str">
+        <x:v>survey-035</x:v>
+      </x:c>
+      <x:c r="F41" s="35"/>
+      <x:c r="G41" s="35"/>
+      <x:c r="H41" s="35"/>
+      <x:c r="I41" s="35"/>
+      <x:c r="J41" s="35"/>
+      <x:c r="K41" s="35"/>
+      <x:c r="L41" s="35"/>
+      <x:c r="M41" s="35"/>
+      <x:c r="N41" s="35"/>
+    </x:row>
+    <x:row r="42">
+      <x:c r="A42" s="39" t="n">
+        <x:v>3167.6544215999998</x:v>
+      </x:c>
+      <x:c r="B42" s="39" t="n">
+        <x:v>1.5399738122046764</x:v>
+      </x:c>
+      <x:c r="C42" s="39" t="n">
+        <x:v>1.0947403200209231</x:v>
+      </x:c>
+      <x:c r="D42" s="39" t="n">
+        <x:v>0.216</x:v>
+      </x:c>
+      <x:c r="E42" s="35" t="str">
+        <x:v>survey-036</x:v>
+      </x:c>
+      <x:c r="F42" s="35"/>
+      <x:c r="G42" s="35"/>
+      <x:c r="H42" s="35"/>
+      <x:c r="I42" s="35"/>
+      <x:c r="J42" s="35"/>
+      <x:c r="K42" s="35"/>
+      <x:c r="L42" s="35"/>
+      <x:c r="M42" s="35"/>
+      <x:c r="N42" s="35"/>
+    </x:row>
+    <x:row r="43">
+      <x:c r="A43" s="39" t="n">
+        <x:v>3243.9723792</x:v>
+      </x:c>
+      <x:c r="B43" s="39" t="n">
+        <x:v>1.5430455916881864</x:v>
+      </x:c>
+      <x:c r="C43" s="39" t="n">
+        <x:v>1.0980389923071925</x:v>
+      </x:c>
+      <x:c r="D43" s="39" t="n">
+        <x:v>0.216</x:v>
+      </x:c>
+      <x:c r="E43" s="35" t="str">
+        <x:v>survey-037</x:v>
+      </x:c>
+      <x:c r="F43" s="35"/>
+      <x:c r="G43" s="35"/>
+      <x:c r="H43" s="35"/>
+      <x:c r="I43" s="35"/>
+      <x:c r="J43" s="35"/>
+      <x:c r="K43" s="35"/>
+      <x:c r="L43" s="35"/>
+      <x:c r="M43" s="35"/>
+      <x:c r="N43" s="35"/>
+    </x:row>
+    <x:row r="44">
+      <x:c r="A44" s="39" t="n">
+        <x:v>3319.6978056000003</x:v>
+      </x:c>
+      <x:c r="B44" s="39" t="n">
+        <x:v>1.5477405273760516</x:v>
+      </x:c>
+      <x:c r="C44" s="39" t="n">
+        <x:v>1.1023848621446584</x:v>
+      </x:c>
+      <x:c r="D44" s="39" t="n">
+        <x:v>0.216</x:v>
+      </x:c>
+      <x:c r="E44" s="35" t="str">
+        <x:v>survey-038</x:v>
+      </x:c>
+      <x:c r="F44" s="35"/>
+      <x:c r="G44" s="35"/>
+      <x:c r="H44" s="35"/>
+      <x:c r="I44" s="35"/>
+      <x:c r="J44" s="35"/>
+      <x:c r="K44" s="35"/>
+      <x:c r="L44" s="35"/>
+      <x:c r="M44" s="35"/>
+      <x:c r="N44" s="35"/>
+    </x:row>
+    <x:row r="45">
+      <x:c r="A45" s="39" t="n">
+        <x:v>3395.1068496000003</x:v>
+      </x:c>
+      <x:c r="B45" s="39" t="n">
+        <x:v>1.5533430342749535</x:v>
+      </x:c>
+      <x:c r="C45" s="39" t="n">
+        <x:v>1.1082840750163994</x:v>
+      </x:c>
+      <x:c r="D45" s="39" t="n">
+        <x:v>0.216</x:v>
+      </x:c>
+      <x:c r="E45" s="35" t="str">
+        <x:v>survey-039</x:v>
+      </x:c>
+      <x:c r="F45" s="35"/>
+      <x:c r="G45" s="35"/>
+      <x:c r="H45" s="35"/>
+      <x:c r="I45" s="35"/>
+      <x:c r="J45" s="35"/>
+      <x:c r="K45" s="35"/>
+      <x:c r="L45" s="35"/>
+      <x:c r="M45" s="35"/>
+      <x:c r="N45" s="35"/>
+    </x:row>
+    <x:row r="46">
+      <x:c r="A46" s="39" t="n">
+        <x:v>3470.6368992</x:v>
+      </x:c>
+      <x:c r="B46" s="39" t="n">
+        <x:v>1.5589455411738549</x:v>
+      </x:c>
+      <x:c r="C46" s="39" t="n">
+        <x:v>1.1161031500653338</x:v>
+      </x:c>
+      <x:c r="D46" s="39" t="n">
+        <x:v>0.216</x:v>
+      </x:c>
+      <x:c r="E46" s="35" t="str">
+        <x:v>survey-040</x:v>
+      </x:c>
+      <x:c r="F46" s="35"/>
+      <x:c r="G46" s="35"/>
+      <x:c r="H46" s="35"/>
+      <x:c r="I46" s="35"/>
+      <x:c r="J46" s="35"/>
+      <x:c r="K46" s="35"/>
+      <x:c r="L46" s="35"/>
+      <x:c r="M46" s="35"/>
+      <x:c r="N46" s="35"/>
+    </x:row>
+    <x:row r="47">
+      <x:c r="A47" s="39" t="n">
+        <x:v>3546.6631632</x:v>
+      </x:c>
+      <x:c r="B47" s="39" t="n">
+        <x:v>1.5636404768617198</x:v>
+      </x:c>
+      <x:c r="C47" s="39" t="n">
+        <x:v>1.1261387932643012</x:v>
+      </x:c>
+      <x:c r="D47" s="39" t="n">
+        <x:v>0.216</x:v>
+      </x:c>
+      <x:c r="E47" s="35" t="str">
+        <x:v>survey-041</x:v>
+      </x:c>
+      <x:c r="F47" s="35"/>
+      <x:c r="G47" s="35"/>
+      <x:c r="H47" s="35"/>
+      <x:c r="I47" s="35"/>
+      <x:c r="J47" s="35"/>
+      <x:c r="K47" s="35"/>
+      <x:c r="L47" s="35"/>
+      <x:c r="M47" s="35"/>
+      <x:c r="N47" s="35"/>
+    </x:row>
+    <x:row r="48">
+      <x:c r="A48" s="39" t="n">
+        <x:v>3623.3087808</x:v>
+      </x:c>
+      <x:c r="B48" s="39" t="n">
+        <x:v>1.5667122563452298</x:v>
+      </x:c>
+      <x:c r="C48" s="39" t="n">
+        <x:v>1.1385480842459808</x:v>
+      </x:c>
+      <x:c r="D48" s="39" t="n">
+        <x:v>0.216</x:v>
+      </x:c>
+      <x:c r="E48" s="35" t="str">
+        <x:v>survey-042</x:v>
+      </x:c>
+      <x:c r="F48" s="35"/>
+      <x:c r="G48" s="35"/>
+      <x:c r="H48" s="35"/>
+      <x:c r="I48" s="35"/>
+      <x:c r="J48" s="35"/>
+      <x:c r="K48" s="35"/>
+      <x:c r="L48" s="35"/>
+      <x:c r="M48" s="35"/>
+      <x:c r="N48" s="35"/>
+    </x:row>
+    <x:row r="49">
+      <x:c r="A49" s="39" t="n">
+        <x:v>3700.3805088</x:v>
+      </x:c>
+      <x:c r="B49" s="39" t="n">
+        <x:v>1.5677943604814664</x:v>
+      </x:c>
+      <x:c r="C49" s="39" t="n">
+        <x:v>1.1534182894729725</x:v>
+      </x:c>
+      <x:c r="D49" s="39" t="n">
+        <x:v>0.216</x:v>
+      </x:c>
+      <x:c r="E49" s="35" t="str">
+        <x:v>survey-043</x:v>
+      </x:c>
+      <x:c r="F49" s="35"/>
+      <x:c r="G49" s="35"/>
+      <x:c r="H49" s="35"/>
+      <x:c r="I49" s="35"/>
+      <x:c r="J49" s="35"/>
+      <x:c r="K49" s="35"/>
+      <x:c r="L49" s="35"/>
+      <x:c r="M49" s="35"/>
+      <x:c r="N49" s="35"/>
+    </x:row>
+    <x:row r="50">
+      <x:c r="A50" s="39" t="n">
+        <x:v>3777.4683912</x:v>
+      </x:c>
+      <x:c r="B50" s="39" t="n">
+        <x:v>1.5669042425629494</x:v>
+      </x:c>
+      <x:c r="C50" s="39" t="n">
+        <x:v>1.1706621424826766</x:v>
+      </x:c>
+      <x:c r="D50" s="39" t="n">
+        <x:v>0.216</x:v>
+      </x:c>
+      <x:c r="E50" s="35" t="str">
+        <x:v>survey-044</x:v>
+      </x:c>
+      <x:c r="F50" s="35"/>
+      <x:c r="G50" s="35"/>
+      <x:c r="H50" s="35"/>
+      <x:c r="I50" s="35"/>
+      <x:c r="J50" s="35"/>
+      <x:c r="K50" s="35"/>
+      <x:c r="L50" s="35"/>
+      <x:c r="M50" s="35"/>
+      <x:c r="N50" s="35"/>
+    </x:row>
+    <x:row r="51">
+      <x:c r="A51" s="39" t="n">
+        <x:v>3854.1542424</x:v>
+      </x:c>
+      <x:c r="B51" s="39" t="n">
+        <x:v>1.5644084217325975</x:v>
+      </x:c>
+      <x:c r="C51" s="39" t="n">
+        <x:v>1.190174923519973</x:v>
+      </x:c>
+      <x:c r="D51" s="39" t="n">
+        <x:v>0.216</x:v>
+      </x:c>
+      <x:c r="E51" s="35" t="str">
+        <x:v>survey-045</x:v>
+      </x:c>
+      <x:c r="F51" s="35"/>
+      <x:c r="G51" s="35"/>
+      <x:c r="H51" s="35"/>
+      <x:c r="I51" s="35"/>
+      <x:c r="J51" s="35"/>
+      <x:c r="K51" s="35"/>
+      <x:c r="L51" s="35"/>
+      <x:c r="M51" s="35"/>
+      <x:c r="N51" s="35"/>
+    </x:row>
+    <x:row r="52">
+      <x:c r="A52" s="39" t="n">
+        <x:v>3930.2240928</x:v>
+      </x:c>
+      <x:c r="B52" s="39" t="n">
+        <x:v>1.5609526698136487</x:v>
+      </x:c>
+      <x:c r="C52" s="39" t="n">
+        <x:v>1.2117297397821032</x:v>
+      </x:c>
+      <x:c r="D52" s="39" t="n">
+        <x:v>0.216</x:v>
+      </x:c>
+      <x:c r="E52" s="35" t="str">
+        <x:v>survey-046</x:v>
+      </x:c>
+      <x:c r="F52" s="35"/>
+      <x:c r="G52" s="35"/>
+      <x:c r="H52" s="35"/>
+      <x:c r="I52" s="35"/>
+      <x:c r="J52" s="35"/>
+      <x:c r="K52" s="35"/>
+      <x:c r="L52" s="35"/>
+      <x:c r="M52" s="35"/>
+      <x:c r="N52" s="35"/>
+    </x:row>
+    <x:row r="53">
+      <x:c r="A53" s="39" t="n">
+        <x:v>4005.779136</x:v>
+      </x:c>
+      <x:c r="B53" s="39" t="n">
+        <x:v>1.5572002119218606</x:v>
+      </x:c>
+      <x:c r="C53" s="39" t="n">
+        <x:v>1.2350473385887475</x:v>
+      </x:c>
+      <x:c r="D53" s="39" t="n">
+        <x:v>0.216</x:v>
+      </x:c>
+      <x:c r="E53" s="35" t="str">
+        <x:v>survey-047</x:v>
+      </x:c>
+      <x:c r="F53" s="35"/>
+      <x:c r="G53" s="35"/>
+      <x:c r="H53" s="35"/>
+      <x:c r="I53" s="35"/>
+      <x:c r="J53" s="35"/>
+      <x:c r="K53" s="35"/>
+      <x:c r="L53" s="35"/>
+      <x:c r="M53" s="35"/>
+      <x:c r="N53" s="35"/>
+    </x:row>
+    <x:row r="54">
+      <x:c r="A54" s="39" t="n">
+        <x:v>4081.1817792</x:v>
+      </x:c>
+      <x:c r="B54" s="39" t="n">
+        <x:v>1.553727006710392</x:v>
+      </x:c>
+      <x:c r="C54" s="39" t="n">
+        <x:v>1.2598135606745469</x:v>
+      </x:c>
+      <x:c r="D54" s="39" t="n">
+        <x:v>0.216</x:v>
+      </x:c>
+      <x:c r="E54" s="35" t="str">
+        <x:v>survey-048</x:v>
+      </x:c>
+      <x:c r="F54" s="35"/>
+      <x:c r="G54" s="35"/>
+      <x:c r="H54" s="35"/>
+      <x:c r="I54" s="35"/>
+      <x:c r="J54" s="35"/>
+      <x:c r="K54" s="35"/>
+      <x:c r="L54" s="35"/>
+      <x:c r="M54" s="35"/>
+      <x:c r="N54" s="35"/>
+    </x:row>
+    <x:row r="55">
+      <x:c r="A55" s="39" t="n">
+        <x:v>4156.8727632</x:v>
+      </x:c>
+      <x:c r="B55" s="39" t="n">
+        <x:v>1.5508821200296412</x:v>
+      </x:c>
+      <x:c r="C55" s="39" t="n">
+        <x:v>1.285679340189103</x:v>
+      </x:c>
+      <x:c r="D55" s="39" t="n">
+        <x:v>0.216</x:v>
+      </x:c>
+      <x:c r="E55" s="35" t="str">
+        <x:v>survey-049</x:v>
+      </x:c>
+      <x:c r="F55" s="35"/>
+      <x:c r="G55" s="35"/>
+      <x:c r="H55" s="35"/>
+      <x:c r="I55" s="35"/>
+      <x:c r="J55" s="35"/>
+      <x:c r="K55" s="35"/>
+      <x:c r="L55" s="35"/>
+      <x:c r="M55" s="35"/>
+      <x:c r="N55" s="35"/>
+    </x:row>
+    <x:row r="56">
+      <x:c r="A56" s="39" t="n">
+        <x:v>4233.1456104</x:v>
+      </x:c>
+      <x:c r="B56" s="39" t="n">
+        <x:v>1.548752818342208</x:v>
+      </x:c>
+      <x:c r="C56" s="39" t="n">
+        <x:v>1.3123479711595762</x:v>
+      </x:c>
+      <x:c r="D56" s="39" t="n">
+        <x:v>0.216</x:v>
+      </x:c>
+      <x:c r="E56" s="35" t="str">
+        <x:v>survey-050</x:v>
+      </x:c>
+      <x:c r="F56" s="35"/>
+      <x:c r="G56" s="35"/>
+      <x:c r="H56" s="35"/>
+      <x:c r="I56" s="35"/>
+      <x:c r="J56" s="35"/>
+      <x:c r="K56" s="35"/>
+      <x:c r="L56" s="35"/>
+      <x:c r="M56" s="35"/>
+      <x:c r="N56" s="35"/>
+    </x:row>
+    <x:row r="57">
+      <x:c r="A57" s="39" t="n">
+        <x:v>4309.9975776</x:v>
+      </x:c>
+      <x:c r="B57" s="39" t="n">
+        <x:v>1.5472343818929732</x:v>
+      </x:c>
+      <x:c r="C57" s="39" t="n">
+        <x:v>1.339487841028088</x:v>
+      </x:c>
+      <x:c r="D57" s="39" t="n">
+        <x:v>0.216</x:v>
+      </x:c>
+      <x:c r="E57" s="35" t="str">
+        <x:v>survey-051</x:v>
+      </x:c>
+      <x:c r="F57" s="35"/>
+      <x:c r="G57" s="35"/>
+      <x:c r="H57" s="35"/>
+      <x:c r="I57" s="35"/>
+      <x:c r="J57" s="35"/>
+      <x:c r="K57" s="35"/>
+      <x:c r="L57" s="35"/>
+      <x:c r="M57" s="35"/>
+      <x:c r="N57" s="35"/>
+    </x:row>
+    <x:row r="58">
+      <x:c r="A58" s="39" t="n">
+        <x:v>4387.1302656</x:v>
+      </x:c>
+      <x:c r="B58" s="39" t="n">
+        <x:v>1.546117371171697</x:v>
+      </x:c>
+      <x:c r="C58" s="39" t="n">
+        <x:v>1.366837150406839</x:v>
+      </x:c>
+      <x:c r="D58" s="39" t="n">
+        <x:v>0.216</x:v>
+      </x:c>
+      <x:c r="E58" s="35" t="str">
+        <x:v>survey-052</x:v>
+      </x:c>
+      <x:c r="F58" s="35"/>
+      <x:c r="G58" s="35"/>
+      <x:c r="H58" s="35"/>
+      <x:c r="I58" s="35"/>
+      <x:c r="J58" s="35"/>
+      <x:c r="K58" s="35"/>
+      <x:c r="L58" s="35"/>
+      <x:c r="M58" s="35"/>
+      <x:c r="N58" s="35"/>
+    </x:row>
+    <x:row r="59">
+      <x:c r="A59" s="39" t="n">
+        <x:v>4464.1026288</x:v>
+      </x:c>
+      <x:c r="B59" s="39" t="n">
+        <x:v>1.54517489337562</x:v>
+      </x:c>
+      <x:c r="C59" s="39" t="n">
+        <x:v>1.3941690064930703</x:v>
+      </x:c>
+      <x:c r="D59" s="39" t="n">
+        <x:v>0.216</x:v>
+      </x:c>
+      <x:c r="E59" s="35" t="str">
+        <x:v>survey-053</x:v>
+      </x:c>
+      <x:c r="F59" s="35"/>
+      <x:c r="G59" s="35"/>
+      <x:c r="H59" s="35"/>
+      <x:c r="I59" s="35"/>
+      <x:c r="J59" s="35"/>
+      <x:c r="K59" s="35"/>
+      <x:c r="L59" s="35"/>
+      <x:c r="M59" s="35"/>
+      <x:c r="N59" s="35"/>
+    </x:row>
+    <x:row r="60">
+      <x:c r="A60" s="39" t="n">
+        <x:v>4540.555308</x:v>
+      </x:c>
+      <x:c r="B60" s="39" t="n">
+        <x:v>1.5443545886271826</x:v>
+      </x:c>
+      <x:c r="C60" s="39" t="n">
+        <x:v>1.421343782946622</x:v>
+      </x:c>
+      <x:c r="D60" s="39" t="n">
+        <x:v>0.216</x:v>
+      </x:c>
+      <x:c r="E60" s="35" t="str">
+        <x:v>survey-054</x:v>
+      </x:c>
+      <x:c r="F60" s="35"/>
+      <x:c r="G60" s="35"/>
+      <x:c r="H60" s="35"/>
+      <x:c r="I60" s="35"/>
+      <x:c r="J60" s="35"/>
+      <x:c r="K60" s="35"/>
+      <x:c r="L60" s="35"/>
+      <x:c r="M60" s="35"/>
+      <x:c r="N60" s="35"/>
+    </x:row>
+    <x:row r="61">
+      <x:c r="A61" s="39" t="n">
+        <x:v>4616.3935104</x:v>
+      </x:c>
+      <x:c r="B61" s="39" t="n">
+        <x:v>1.5437786299740244</x:v>
+      </x:c>
+      <x:c r="C61" s="39" t="n">
+        <x:v>1.4482567600123746</x:v>
+      </x:c>
+      <x:c r="D61" s="39" t="n">
+        <x:v>0.216</x:v>
+      </x:c>
+      <x:c r="E61" s="35" t="str">
+        <x:v>survey-055</x:v>
+      </x:c>
+      <x:c r="F61" s="35"/>
+      <x:c r="G61" s="35"/>
+      <x:c r="H61" s="35"/>
+      <x:c r="I61" s="35"/>
+      <x:c r="J61" s="35"/>
+      <x:c r="K61" s="35"/>
+      <x:c r="L61" s="35"/>
+      <x:c r="M61" s="35"/>
+      <x:c r="N61" s="35"/>
+    </x:row>
+    <x:row r="62">
+      <x:c r="A62" s="39" t="n">
+        <x:v>4691.8360824</x:v>
+      </x:c>
+      <x:c r="B62" s="39" t="n">
+        <x:v>1.5437262700964647</x:v>
+      </x:c>
+      <x:c r="C62" s="39" t="n">
+        <x:v>1.4748730311052882</x:v>
+      </x:c>
+      <x:c r="D62" s="39" t="n">
+        <x:v>0.216</x:v>
+      </x:c>
+      <x:c r="E62" s="35" t="str">
+        <x:v>survey-056</x:v>
+      </x:c>
+      <x:c r="F62" s="35"/>
+      <x:c r="G62" s="35"/>
+      <x:c r="H62" s="35"/>
+      <x:c r="I62" s="35"/>
+      <x:c r="J62" s="35"/>
+      <x:c r="K62" s="35"/>
+      <x:c r="L62" s="35"/>
+      <x:c r="M62" s="35"/>
+      <x:c r="N62" s="35"/>
+    </x:row>
+    <x:row r="63">
+      <x:c r="A63" s="39" t="n">
+        <x:v>4767.3027336000005</x:v>
+      </x:c>
+      <x:c r="B63" s="39" t="n">
+        <x:v>1.5445814814299417</x:v>
+      </x:c>
+      <x:c r="C63" s="39" t="n">
+        <x:v>1.5012100495178828</x:v>
+      </x:c>
+      <x:c r="D63" s="39" t="n">
+        <x:v>0.216</x:v>
+      </x:c>
+      <x:c r="E63" s="35" t="str">
+        <x:v>survey-057</x:v>
+      </x:c>
+      <x:c r="F63" s="35"/>
+      <x:c r="G63" s="35"/>
+      <x:c r="H63" s="35"/>
+      <x:c r="I63" s="35"/>
+      <x:c r="J63" s="35"/>
+      <x:c r="K63" s="35"/>
+      <x:c r="L63" s="35"/>
+      <x:c r="M63" s="35"/>
+      <x:c r="N63" s="35"/>
+    </x:row>
+    <x:row r="64">
+      <x:c r="A64" s="39" t="n">
+        <x:v>4843.2018960000005</x:v>
+      </x:c>
+      <x:c r="B64" s="39" t="n">
+        <x:v>1.5465886100697352</x:v>
+      </x:c>
+      <x:c r="C64" s="39" t="n">
+        <x:v>1.5273376284202378</x:v>
+      </x:c>
+      <x:c r="D64" s="39" t="n">
+        <x:v>0.216</x:v>
+      </x:c>
+      <x:c r="E64" s="35" t="str">
+        <x:v>survey-058</x:v>
+      </x:c>
+      <x:c r="F64" s="35"/>
+      <x:c r="G64" s="35"/>
+      <x:c r="H64" s="35"/>
+      <x:c r="I64" s="35"/>
+      <x:c r="J64" s="35"/>
+      <x:c r="K64" s="35"/>
+      <x:c r="L64" s="35"/>
+      <x:c r="M64" s="35"/>
+      <x:c r="N64" s="35"/>
+    </x:row>
+    <x:row r="65">
+      <x:c r="A65" s="39" t="n">
+        <x:v>4919.7207168</x:v>
+      </x:c>
+      <x:c r="B65" s="39" t="n">
+        <x:v>1.5498523757709646</x:v>
+      </x:c>
+      <x:c r="C65" s="39" t="n">
+        <x:v>1.5533430342749535</x:v>
+      </x:c>
+      <x:c r="D65" s="39" t="n">
+        <x:v>0.216</x:v>
+      </x:c>
+      <x:c r="E65" s="35" t="str">
+        <x:v>survey-059</x:v>
+      </x:c>
+      <x:c r="F65" s="35"/>
+      <x:c r="G65" s="35"/>
+      <x:c r="H65" s="35"/>
+      <x:c r="I65" s="35"/>
+      <x:c r="J65" s="35"/>
+      <x:c r="K65" s="35"/>
+      <x:c r="L65" s="35"/>
+      <x:c r="M65" s="35"/>
+      <x:c r="N65" s="35"/>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:N1"/>
+    <x:mergeCell ref="A3:F3"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -11812,11 +13971,11 @@
       </x:c>
       <x:c r="B10" s="37" t="n">
         <x:f>Inputs!B14*'Unit Map'!$I$13</x:f>
-        <x:v>1400</x:v>
+        <x:v>1.4000000000000001</x:v>
       </x:c>
       <x:c r="C10" s="37" t="str">
         <x:f>'Unit Map'!$H$13</x:f>
-        <x:v>kg/m3</x:v>
+        <x:v>g/cm3</x:v>
       </x:c>
       <x:c r="D10" s="37" t="str">
         <x:v>Screening only</x:v>
@@ -14449,7 +16608,7 @@
       </x:c>
       <x:c r="H5" s="36" t="str">
         <x:f>"ECD "&amp;'Unit Map'!$H$13</x:f>
-        <x:v>ECD kg/m3</x:v>
+        <x:v>ECD g/cm3</x:v>
       </x:c>
       <x:c r="I5" s="36" t="str">
         <x:v>Pressure % limit</x:v>
@@ -14493,7 +16652,7 @@
       </x:c>
       <x:c r="H6" s="37" t="n">
         <x:f>('Inputs'!$B$9+IF('Inputs'!G6="Annulus",'Calc'!G6/(9.80665*MAX('Calc'!B6,1)),0))*'Unit Map'!$I$13</x:f>
-        <x:v>1200</x:v>
+        <x:v>1.2</x:v>
       </x:c>
       <x:c r="I6" s="37" t="n">
         <x:f>'Calc'!H6/'Inputs'!$B$6</x:f>
@@ -14539,7 +16698,7 @@
       </x:c>
       <x:c r="H7" s="37" t="n">
         <x:f>('Inputs'!$B$9+IF('Inputs'!G7="Annulus",'Calc'!G7/(9.80665*MAX('Calc'!B7,1)),0))*'Unit Map'!$I$13</x:f>
-        <x:v>1200</x:v>
+        <x:v>1.2</x:v>
       </x:c>
       <x:c r="I7" s="37" t="n">
         <x:f>'Calc'!H7/'Inputs'!$B$6</x:f>
@@ -14585,7 +16744,7 @@
       </x:c>
       <x:c r="H8" s="37" t="n">
         <x:f>('Inputs'!$B$9+IF('Inputs'!G8="Annulus",'Calc'!G8/(9.80665*MAX('Calc'!B8,1)),0))*'Unit Map'!$I$13</x:f>
-        <x:v>1200</x:v>
+        <x:v>1.2</x:v>
       </x:c>
       <x:c r="I8" s="37" t="n">
         <x:f>'Calc'!H8/'Inputs'!$B$6</x:f>
@@ -14631,7 +16790,7 @@
       </x:c>
       <x:c r="H9" s="37" t="n">
         <x:f>('Inputs'!$B$9+IF('Inputs'!G9="Annulus",'Calc'!G9/(9.80665*MAX('Calc'!B9,1)),0))*'Unit Map'!$I$13</x:f>
-        <x:v>1200</x:v>
+        <x:v>1.2</x:v>
       </x:c>
       <x:c r="I9" s="37" t="n">
         <x:f>'Calc'!H9/'Inputs'!$B$6</x:f>
@@ -14677,7 +16836,7 @@
       </x:c>
       <x:c r="H10" s="37" t="n">
         <x:f>('Inputs'!$B$9+IF('Inputs'!G10="Annulus",'Calc'!G10/(9.80665*MAX('Calc'!B10,1)),0))*'Unit Map'!$I$13</x:f>
-        <x:v>1200</x:v>
+        <x:v>1.2</x:v>
       </x:c>
       <x:c r="I10" s="37" t="n">
         <x:f>'Calc'!H10/'Inputs'!$B$6</x:f>
@@ -14723,7 +16882,7 @@
       </x:c>
       <x:c r="H11" s="37" t="n">
         <x:f>('Inputs'!$B$9+IF('Inputs'!G11="Annulus",'Calc'!G11/(9.80665*MAX('Calc'!B11,1)),0))*'Unit Map'!$I$13</x:f>
-        <x:v>1200</x:v>
+        <x:v>1.2</x:v>
       </x:c>
       <x:c r="I11" s="37" t="n">
         <x:f>'Calc'!H11/'Inputs'!$B$6</x:f>
@@ -14769,7 +16928,7 @@
       </x:c>
       <x:c r="H12" s="37" t="n">
         <x:f>('Inputs'!$B$9+IF('Inputs'!G12="Annulus",'Calc'!G12/(9.80665*MAX('Calc'!B12,1)),0))*'Unit Map'!$I$13</x:f>
-        <x:v>1200</x:v>
+        <x:v>1.2</x:v>
       </x:c>
       <x:c r="I12" s="37" t="n">
         <x:f>'Calc'!H12/'Inputs'!$B$6</x:f>
@@ -14815,7 +16974,7 @@
       </x:c>
       <x:c r="H13" s="37" t="n">
         <x:f>('Inputs'!$B$9+IF('Inputs'!G13="Annulus",'Calc'!G13/(9.80665*MAX('Calc'!B13,1)),0))*'Unit Map'!$I$13</x:f>
-        <x:v>1769.9514042766855</x:v>
+        <x:v>1.7699514042766855</x:v>
       </x:c>
       <x:c r="I13" s="37" t="n">
         <x:f>'Calc'!H13/'Inputs'!$B$6</x:f>

</xml_diff>